<commit_message>
final upload after completing the research project
</commit_message>
<xml_diff>
--- a/smoothed_signal.xlsx
+++ b/smoothed_signal.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Linear Model\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F261C63E-8835-4734-9E52-703D4A80C406}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -70,11 +64,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -138,21 +132,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -190,7 +176,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -224,7 +210,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -259,10 +244,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -435,16 +419,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O70"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="26.77734375" customWidth="1"/>
-    <col min="14" max="14" width="22.21875" customWidth="1"/>
-    <col min="15" max="15" width="22.109375" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -491,27 +470,27 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15">
       <c r="A2" s="2">
         <v>43833</v>
       </c>
       <c r="B2">
-        <v>1.0508276937125289E-2</v>
+        <v>0.01050827693712529</v>
       </c>
       <c r="C2">
-        <v>1.2100658749178671E-3</v>
+        <v>0.001210065874917867</v>
       </c>
       <c r="D2">
-        <v>2.200501696373766E-3</v>
+        <v>0.002200501696373766</v>
       </c>
       <c r="E2">
         <v>0.1204356613057983</v>
       </c>
       <c r="F2">
-        <v>-7.8286199376013138E-2</v>
+        <v>-0.07828619937601314</v>
       </c>
       <c r="G2">
-        <v>8.5225755263597935E-3</v>
+        <v>0.008522575526359794</v>
       </c>
       <c r="H2">
         <v>14</v>
@@ -523,13 +502,13 @@
         <v>3.630639893011828</v>
       </c>
       <c r="K2">
-        <v>0.28115219958952481</v>
+        <v>0.2811521995895248</v>
       </c>
       <c r="L2">
-        <v>4.3797571450936426</v>
+        <v>4.379757145093643</v>
       </c>
       <c r="M2">
-        <v>-1.339888319410347E-2</v>
+        <v>-0.01339888319410347</v>
       </c>
       <c r="N2">
         <v>0.1944091721008876</v>
@@ -538,27 +517,27 @@
         <v>0.2186350552298493</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15">
       <c r="A3" s="2">
         <v>43862</v>
       </c>
       <c r="B3">
-        <v>1.068787063672373E-2</v>
+        <v>0.01068787063672373</v>
       </c>
       <c r="C3">
-        <v>-8.6040523437962201E-5</v>
+        <v>-8.60405234379622E-05</v>
       </c>
       <c r="D3">
-        <v>2.4459907620128811E-3</v>
+        <v>0.002445990762012881</v>
       </c>
       <c r="E3">
-        <v>-9.4758165097150765E-2</v>
+        <v>-0.09475816509715076</v>
       </c>
       <c r="F3">
-        <v>-0.55803624576923072</v>
+        <v>-0.5580362457692307</v>
       </c>
       <c r="G3">
-        <v>1.290292850575284E-2</v>
+        <v>0.01290292850575284</v>
       </c>
       <c r="H3">
         <v>15</v>
@@ -567,45 +546,45 @@
         <v>19</v>
       </c>
       <c r="J3">
-        <v>4.3117887220864404</v>
+        <v>4.31178872208644</v>
       </c>
       <c r="K3">
-        <v>0.41566738259504288</v>
+        <v>0.4156673825950429</v>
       </c>
       <c r="L3">
-        <v>7.3011347355978051</v>
+        <v>7.301134735597805</v>
       </c>
       <c r="M3">
-        <v>-3.5111796304096443E-2</v>
+        <v>-0.03511179630409644</v>
       </c>
       <c r="N3">
-        <v>0.24881388523116629</v>
+        <v>0.2488138852311663</v>
       </c>
       <c r="O3">
-        <v>0.23876229158774809</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.2387622915877481</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15">
       <c r="A4" s="2">
         <v>43896</v>
       </c>
       <c r="B4">
-        <v>1.4533672847002641E-2</v>
+        <v>0.01453367284700264</v>
       </c>
       <c r="C4">
-        <v>1.125260342018636E-3</v>
+        <v>0.001125260342018636</v>
       </c>
       <c r="D4">
-        <v>5.588541095654348E-3</v>
+        <v>0.005588541095654348</v>
       </c>
       <c r="E4">
         <v>-0.1213824728544312</v>
       </c>
       <c r="F4">
-        <v>-0.30189071620766839</v>
+        <v>-0.3018907162076684</v>
       </c>
       <c r="G4">
-        <v>4.3536297280413958E-2</v>
+        <v>0.04353629728041396</v>
       </c>
       <c r="H4">
         <v>22</v>
@@ -617,42 +596,42 @@
         <v>3.638416490038773</v>
       </c>
       <c r="K4">
-        <v>0.28268794380222639</v>
+        <v>0.2826879438022264</v>
       </c>
       <c r="L4">
-        <v>8.6227784518542183</v>
+        <v>8.622778451854218</v>
       </c>
       <c r="M4">
-        <v>-3.9220854643383173E-2</v>
+        <v>-0.03922085464338317</v>
       </c>
       <c r="N4">
-        <v>0.37309632334446569</v>
+        <v>0.3730963233444657</v>
       </c>
       <c r="O4">
-        <v>0.30995559804517581</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.3099555980451758</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15">
       <c r="A5" s="2">
         <v>43924</v>
       </c>
       <c r="B5">
-        <v>1.697196585759143E-2</v>
+        <v>0.01697196585759143</v>
       </c>
       <c r="C5">
-        <v>-7.8212426577286751E-4</v>
+        <v>-0.0007821242657728675</v>
       </c>
       <c r="D5">
-        <v>7.1058690237439954E-3</v>
+        <v>0.007105869023743995</v>
       </c>
       <c r="E5">
-        <v>-6.573053834558433E-2</v>
+        <v>-0.06573053834558433</v>
       </c>
       <c r="F5">
         <v>-0.2231387967401279</v>
       </c>
       <c r="G5">
-        <v>2.0059790833634461E-2</v>
+        <v>0.02005979083363446</v>
       </c>
       <c r="H5">
         <v>24</v>
@@ -661,45 +640,45 @@
         <v>27</v>
       </c>
       <c r="J5">
-        <v>2.9685765523023422</v>
+        <v>2.968576552302342</v>
       </c>
       <c r="K5">
-        <v>0.12686826555654021</v>
+        <v>0.1268682655565402</v>
       </c>
       <c r="L5">
-        <v>19.683180316277259</v>
+        <v>19.68318031627726</v>
       </c>
       <c r="M5">
-        <v>-7.882007989160203E-2</v>
+        <v>-0.07882007989160203</v>
       </c>
       <c r="N5">
-        <v>0.46198366139175812</v>
+        <v>0.4619836613917581</v>
       </c>
       <c r="O5">
-        <v>0.35647117282415491</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.3564711728241549</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15">
       <c r="A6" s="2">
         <v>43959</v>
       </c>
       <c r="B6">
-        <v>1.6027821747770669E-2</v>
+        <v>0.01602782174777067</v>
       </c>
       <c r="C6">
-        <v>4.5213780164144889E-4</v>
+        <v>0.0004521378016414489</v>
       </c>
       <c r="D6">
-        <v>5.7947762610165406E-3</v>
+        <v>0.005794776261016541</v>
       </c>
       <c r="E6">
-        <v>0.14939783591233111</v>
+        <v>0.1493978359123311</v>
       </c>
       <c r="F6">
         <v>-0.1326760821365611</v>
       </c>
       <c r="G6">
-        <v>1.6468045444791489E-2</v>
+        <v>0.01646804544479149</v>
       </c>
       <c r="H6">
         <v>23</v>
@@ -708,45 +687,45 @@
         <v>24</v>
       </c>
       <c r="J6">
-        <v>4.4315916127633974</v>
+        <v>4.431591612763397</v>
       </c>
       <c r="K6">
         <v>0.370573984813171</v>
       </c>
       <c r="L6">
-        <v>16.775968769631799</v>
+        <v>16.7759687696318</v>
       </c>
       <c r="M6">
-        <v>-5.7877766605356908E-2</v>
+        <v>-0.05787776660535691</v>
       </c>
       <c r="N6">
-        <v>0.32344017343098169</v>
+        <v>0.3234401734309817</v>
       </c>
       <c r="O6">
-        <v>0.33328135228526262</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.3332813522852626</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15">
       <c r="A7" s="2">
         <v>43987</v>
       </c>
       <c r="B7">
-        <v>1.293341873215929E-2</v>
+        <v>0.01293341873215929</v>
       </c>
       <c r="C7">
-        <v>-3.5469467188048659E-4</v>
+        <v>-0.0003546946718804866</v>
       </c>
       <c r="D7">
-        <v>3.776245779582943E-3</v>
+        <v>0.003776245779582943</v>
       </c>
       <c r="E7">
-        <v>-0.13994882963249891</v>
+        <v>-0.1399488296324989</v>
       </c>
       <c r="F7">
-        <v>-0.66235664054532295</v>
+        <v>-0.6623566405453229</v>
       </c>
       <c r="G7">
-        <v>1.207763304234907E-2</v>
+        <v>0.01207763304234907</v>
       </c>
       <c r="H7">
         <v>19</v>
@@ -755,45 +734,45 @@
         <v>17</v>
       </c>
       <c r="J7">
-        <v>5.7207199000105096</v>
+        <v>5.72071990001051</v>
       </c>
       <c r="K7">
-        <v>0.58531404111759422</v>
+        <v>0.5853140411175942</v>
       </c>
       <c r="L7">
-        <v>16.293143900660631</v>
+        <v>16.29314390066063</v>
       </c>
       <c r="M7">
-        <v>-5.508682871676282E-2</v>
+        <v>-0.05508682871676282</v>
       </c>
       <c r="N7">
-        <v>0.57357829555221085</v>
+        <v>0.5735782955522108</v>
       </c>
       <c r="O7">
-        <v>0.44872673087760118</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.4487267308776012</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15">
       <c r="A8" s="2">
         <v>44015</v>
       </c>
       <c r="B8">
-        <v>8.8513948167341233E-3</v>
+        <v>0.008851394816734123</v>
       </c>
       <c r="C8">
-        <v>1.7710136170044399E-4</v>
+        <v>0.000177101361700444</v>
       </c>
       <c r="D8">
-        <v>1.6363363679525701E-3</v>
+        <v>0.00163633636795257</v>
       </c>
       <c r="E8">
         <v>-0.2001617669171871</v>
       </c>
       <c r="F8">
-        <v>-0.25271070012318769</v>
+        <v>-0.2527107001231877</v>
       </c>
       <c r="G8">
-        <v>1.009574003680986E-2</v>
+        <v>0.01009574003680986</v>
       </c>
       <c r="H8">
         <v>9</v>
@@ -802,45 +781,45 @@
         <v>13</v>
       </c>
       <c r="J8">
-        <v>9.8535827095840389</v>
+        <v>9.853582709584039</v>
       </c>
       <c r="K8">
         <v>1</v>
       </c>
       <c r="L8">
-        <v>13.967902388648421</v>
+        <v>13.96790238864842</v>
       </c>
       <c r="M8">
-        <v>-3.8769654994181259E-2</v>
+        <v>-0.03876965499418126</v>
       </c>
       <c r="N8">
-        <v>0.81473321784897956</v>
+        <v>0.8147332178489796</v>
       </c>
       <c r="O8">
-        <v>0.63477617413337128</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.6347761741333713</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15">
       <c r="A9" s="2">
         <v>44050</v>
       </c>
       <c r="B9">
-        <v>1.416932210784877E-2</v>
+        <v>0.01416932210784877</v>
       </c>
       <c r="C9">
-        <v>3.065316216925692E-3</v>
+        <v>0.003065316216925692</v>
       </c>
       <c r="D9">
-        <v>4.2747090588847181E-3</v>
+        <v>0.004274709058884718</v>
       </c>
       <c r="E9">
-        <v>0.47242345526908808</v>
+        <v>0.4724234552690881</v>
       </c>
       <c r="F9">
-        <v>0.14603747555960159</v>
+        <v>0.1460374755596016</v>
       </c>
       <c r="G9">
-        <v>8.8026321787316071E-3</v>
+        <v>0.008802632178731607</v>
       </c>
       <c r="H9">
         <v>21</v>
@@ -849,16 +828,16 @@
         <v>9</v>
       </c>
       <c r="J9">
-        <v>6.4760509676637223</v>
+        <v>6.476050967663722</v>
       </c>
       <c r="K9">
-        <v>0.55829755181831675</v>
+        <v>0.5582975518183168</v>
       </c>
       <c r="L9">
-        <v>11.294668160524591</v>
+        <v>11.29466816052459</v>
       </c>
       <c r="M9">
-        <v>-2.6486660197172988E-2</v>
+        <v>-0.02648666019717299</v>
       </c>
       <c r="N9">
         <v>0.5977039093642087</v>
@@ -867,27 +846,27 @@
         <v>0.6046825919451928</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15">
       <c r="A10" s="2">
         <v>44078</v>
       </c>
       <c r="B10">
-        <v>1.4739529261322919E-2</v>
+        <v>0.01473952926132292</v>
       </c>
       <c r="C10">
-        <v>3.1063268955721359E-3</v>
+        <v>0.003106326895572136</v>
       </c>
       <c r="D10">
-        <v>4.7134319874929352E-3</v>
+        <v>0.004713431987492935</v>
       </c>
       <c r="E10">
-        <v>-0.37343489666854951</v>
+        <v>-0.3734348966685495</v>
       </c>
       <c r="F10">
-        <v>-0.17261697504944931</v>
+        <v>-0.1726169750494493</v>
       </c>
       <c r="G10">
-        <v>1.29422501916401E-2</v>
+        <v>0.0129422501916401</v>
       </c>
       <c r="H10">
         <v>22</v>
@@ -899,42 +878,42 @@
         <v>6.657296570697004</v>
       </c>
       <c r="K10">
-        <v>0.58200025328765936</v>
+        <v>0.5820002532876594</v>
       </c>
       <c r="L10">
         <v>11.50068804838831</v>
       </c>
       <c r="M10">
-        <v>-2.484969918388634E-2</v>
+        <v>-0.02484969918388634</v>
       </c>
       <c r="N10">
-        <v>0.67502292591876834</v>
+        <v>0.6750229259187683</v>
       </c>
       <c r="O10">
-        <v>0.63986485004067661</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.6398648500406766</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15">
       <c r="A11" s="2">
         <v>44105</v>
       </c>
       <c r="B11">
-        <v>8.9956729331350793E-3</v>
+        <v>0.008995672933135079</v>
       </c>
       <c r="C11">
-        <v>3.0172667849716578E-4</v>
+        <v>0.0003017266784971658</v>
       </c>
       <c r="D11">
-        <v>1.7215605088208631E-3</v>
+        <v>0.001721560508820863</v>
       </c>
       <c r="E11">
-        <v>9.0946769841357619E-2</v>
+        <v>0.09094676984135762</v>
       </c>
       <c r="F11">
-        <v>-0.56507579950630538</v>
+        <v>-0.5650757995063054</v>
       </c>
       <c r="G11">
-        <v>9.4761114245371716E-3</v>
+        <v>0.009476111424537172</v>
       </c>
       <c r="H11">
         <v>10</v>
@@ -943,45 +922,45 @@
         <v>11</v>
       </c>
       <c r="J11">
-        <v>9.0529469461288308</v>
+        <v>9.052946946128831</v>
       </c>
       <c r="K11">
-        <v>0.89529549865343061</v>
+        <v>0.8952954986534306</v>
       </c>
       <c r="L11">
-        <v>11.299588552117241</v>
+        <v>11.29958855211724</v>
       </c>
       <c r="M11">
-        <v>-2.2167597962574181E-2</v>
+        <v>-0.02216759796257418</v>
       </c>
       <c r="N11">
-        <v>0.74774500618698836</v>
+        <v>0.7477450061869884</v>
       </c>
       <c r="O11">
         <v>0.697696634604553</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15">
       <c r="A12" s="2">
         <v>44141</v>
       </c>
       <c r="B12">
-        <v>1.0385650169689229E-2</v>
+        <v>0.01038565016968923</v>
       </c>
       <c r="C12">
-        <v>1.015079946427121E-3</v>
+        <v>0.001015079946427121</v>
       </c>
       <c r="D12">
-        <v>2.283800792073974E-3</v>
+        <v>0.002283800792073974</v>
       </c>
       <c r="E12">
         <v>0.1010902936179167</v>
       </c>
       <c r="F12">
-        <v>0.15207061797109869</v>
+        <v>0.1520706179710987</v>
       </c>
       <c r="G12">
-        <v>7.8973999477856931E-3</v>
+        <v>0.007897399947785693</v>
       </c>
       <c r="H12">
         <v>14</v>
@@ -990,45 +969,45 @@
         <v>7</v>
       </c>
       <c r="J12">
-        <v>8.6986676708322079</v>
+        <v>8.698667670832208</v>
       </c>
       <c r="K12">
-        <v>0.84896402490402934</v>
+        <v>0.8489640249040293</v>
       </c>
       <c r="L12">
         <v>12.01846899718648</v>
       </c>
       <c r="M12">
-        <v>-2.309104836162627E-2</v>
+        <v>-0.02309104836162627</v>
       </c>
       <c r="N12">
-        <v>0.73216815831615778</v>
+        <v>0.7321681583161578</v>
       </c>
       <c r="O12">
-        <v>0.72410267764650305</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.724102677646503</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15">
       <c r="A13" s="2">
         <v>44169</v>
       </c>
       <c r="B13">
-        <v>1.3493657295487989E-2</v>
+        <v>0.01349365729548799</v>
       </c>
       <c r="C13">
-        <v>-2.8351980151686461E-5</v>
+        <v>-2.835198015168646E-05</v>
       </c>
       <c r="D13">
-        <v>4.1397130546690789E-3</v>
+        <v>0.004139713054669079</v>
       </c>
       <c r="E13">
         <v>-0.2898950183538973</v>
       </c>
       <c r="F13">
-        <v>-0.58121020929922607</v>
+        <v>-0.5812102092992261</v>
       </c>
       <c r="G13">
-        <v>9.3075229020331569E-3</v>
+        <v>0.009307522902033157</v>
       </c>
       <c r="H13">
         <v>20</v>
@@ -1037,45 +1016,45 @@
         <v>11</v>
       </c>
       <c r="J13">
-        <v>7.9635004241625724</v>
+        <v>7.963500424162572</v>
       </c>
       <c r="K13">
-        <v>0.75282127999755477</v>
+        <v>0.7528212799975548</v>
       </c>
       <c r="L13">
-        <v>11.788713897942671</v>
+        <v>11.78871389794267</v>
       </c>
       <c r="M13">
-        <v>-1.9613698474108751E-2</v>
+        <v>-0.01961369847410875</v>
       </c>
       <c r="N13">
-        <v>0.71451151011481162</v>
+        <v>0.7145115101148116</v>
       </c>
       <c r="O13">
-        <v>0.71974959855980802</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.719749598559808</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15">
       <c r="A14" s="2">
         <v>44197</v>
       </c>
       <c r="B14">
-        <v>1.063632894510036E-2</v>
+        <v>0.01063632894510036</v>
       </c>
       <c r="C14">
-        <v>1.660946143061133E-3</v>
+        <v>0.001660946143061133</v>
       </c>
       <c r="D14">
-        <v>2.5318134486042232E-3</v>
+        <v>0.002531813448604223</v>
       </c>
       <c r="E14">
-        <v>-0.18201686215961671</v>
+        <v>-0.1820168621596167</v>
       </c>
       <c r="F14">
-        <v>-0.36912853265089929</v>
+        <v>-0.3691285326508993</v>
       </c>
       <c r="G14">
-        <v>1.525726748513408E-2</v>
+        <v>0.01525726748513408</v>
       </c>
       <c r="H14">
         <v>14</v>
@@ -1084,45 +1063,45 @@
         <v>22</v>
       </c>
       <c r="J14">
-        <v>9.0262586909520639</v>
+        <v>9.026258690952064</v>
       </c>
       <c r="K14">
-        <v>0.89180529676932541</v>
+        <v>0.8918052967693254</v>
       </c>
       <c r="L14">
         <v>11.82941498252382</v>
       </c>
       <c r="M14">
-        <v>-1.9317947364640441E-2</v>
+        <v>-0.01931794736464044</v>
       </c>
       <c r="N14">
-        <v>0.78815228930920189</v>
+        <v>0.7881522893092019</v>
       </c>
       <c r="O14">
-        <v>0.75789849016795507</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.7578984901679551</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15">
       <c r="A15" s="2">
         <v>44232</v>
       </c>
       <c r="B15">
-        <v>1.4550188010147789E-2</v>
+        <v>0.01455018801014779</v>
       </c>
       <c r="C15">
-        <v>-1.8810204131587479E-4</v>
+        <v>-0.0001881020413158748</v>
       </c>
       <c r="D15">
-        <v>5.5474901530081534E-3</v>
+        <v>0.005547490153008153</v>
       </c>
       <c r="E15">
-        <v>-6.1812847422420519E-2</v>
+        <v>-0.06181284742242052</v>
       </c>
       <c r="F15">
-        <v>-0.41309542729466409</v>
+        <v>-0.4130954272946641</v>
       </c>
       <c r="G15">
-        <v>1.4100938701930729E-2</v>
+        <v>0.01410093870193073</v>
       </c>
       <c r="H15">
         <v>22</v>
@@ -1131,45 +1110,45 @@
         <v>21</v>
       </c>
       <c r="J15">
-        <v>7.8895034784748423</v>
+        <v>7.889503478474842</v>
       </c>
       <c r="K15">
-        <v>0.74314420378756063</v>
+        <v>0.7431442037875606</v>
       </c>
       <c r="L15">
-        <v>12.538797846478021</v>
+        <v>12.53879784647802</v>
       </c>
       <c r="M15">
-        <v>-2.1058839213840771E-2</v>
+        <v>-0.02105883921384077</v>
       </c>
       <c r="N15">
-        <v>0.82339958561306636</v>
+        <v>0.8233995856130664</v>
       </c>
       <c r="O15">
-        <v>0.79068034450415225</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.7906803445041523</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15">
       <c r="A16" s="2">
         <v>44260</v>
       </c>
       <c r="B16">
-        <v>1.5850157060680981E-2</v>
+        <v>0.01585015706068098</v>
       </c>
       <c r="C16">
-        <v>-4.8307712721965771E-4</v>
+        <v>-0.0004830771272196577</v>
       </c>
       <c r="D16">
-        <v>5.9529573460532139E-3</v>
+        <v>0.005952957346053214</v>
       </c>
       <c r="E16">
-        <v>0.33963528004483828</v>
+        <v>0.3396352800448383</v>
       </c>
       <c r="F16">
-        <v>0.57864994049733942</v>
+        <v>0.5786499404973394</v>
       </c>
       <c r="G16">
-        <v>1.239827684537256E-2</v>
+        <v>0.01239827684537256</v>
       </c>
       <c r="H16">
         <v>23</v>
@@ -1178,45 +1157,45 @@
         <v>18</v>
       </c>
       <c r="J16">
-        <v>8.4329849257115743</v>
+        <v>8.432984925711574</v>
       </c>
       <c r="K16">
-        <v>0.81421891281436698</v>
+        <v>0.814218912814367</v>
       </c>
       <c r="L16">
         <v>11.50044811330503</v>
       </c>
       <c r="M16">
-        <v>-1.3488487301267929E-2</v>
+        <v>-0.01348848730126793</v>
       </c>
       <c r="N16">
-        <v>0.81802108870405321</v>
+        <v>0.8180210887040532</v>
       </c>
       <c r="O16">
-        <v>0.80170317125057922</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.8017031712505792</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15">
       <c r="A17" s="2">
         <v>44287</v>
       </c>
       <c r="B17">
-        <v>1.1667532841457421E-2</v>
+        <v>0.01166753284145742</v>
       </c>
       <c r="C17">
-        <v>-3.0394289115331387E-4</v>
+        <v>-0.0003039428911533139</v>
       </c>
       <c r="D17">
-        <v>3.035631454304574E-3</v>
+        <v>0.003035631454304574</v>
       </c>
       <c r="E17">
-        <v>-0.22590514153895411</v>
+        <v>-0.2259051415389541</v>
       </c>
       <c r="F17">
-        <v>-0.16117813223557839</v>
+        <v>-0.1611781322355784</v>
       </c>
       <c r="G17">
-        <v>1.3117914521815099E-2</v>
+        <v>0.0131179145218151</v>
       </c>
       <c r="H17">
         <v>17</v>
@@ -1225,45 +1204,45 @@
         <v>19</v>
       </c>
       <c r="J17">
-        <v>9.6434696917035776</v>
+        <v>9.643469691703578</v>
       </c>
       <c r="K17">
-        <v>0.97252211334070982</v>
+        <v>0.9725221133407098</v>
       </c>
       <c r="L17">
-        <v>10.587564880829699</v>
+        <v>10.5875648808297</v>
       </c>
       <c r="M17">
-        <v>-5.494071625244931E-3</v>
+        <v>-0.005494071625244931</v>
       </c>
       <c r="N17">
-        <v>0.92391801986756839</v>
+        <v>0.9239180198675684</v>
       </c>
       <c r="O17">
-        <v>0.86407429589181461</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.8640742958918146</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15">
       <c r="A18" s="2">
         <v>44323</v>
       </c>
       <c r="B18">
-        <v>1.1153934605991289E-2</v>
+        <v>0.01115393460599129</v>
       </c>
       <c r="C18">
-        <v>2.4198469605106578E-3</v>
+        <v>0.002419846960510658</v>
       </c>
       <c r="D18">
-        <v>2.7688429116749839E-3</v>
+        <v>0.002768842911674984</v>
       </c>
       <c r="E18">
-        <v>-0.15545026738719811</v>
+        <v>-0.1554502673871981</v>
       </c>
       <c r="F18">
-        <v>-0.31067694379365268</v>
+        <v>-0.3106769437936527</v>
       </c>
       <c r="G18">
-        <v>7.8567403970522705E-3</v>
+        <v>0.00785674039705227</v>
       </c>
       <c r="H18">
         <v>16</v>
@@ -1272,45 +1251,45 @@
         <v>7</v>
       </c>
       <c r="J18">
-        <v>9.9274130117242354</v>
+        <v>9.927413011724235</v>
       </c>
       <c r="K18">
-        <v>0.97036627215312921</v>
+        <v>0.9703662721531292</v>
       </c>
       <c r="L18">
-        <v>9.7317824966085116</v>
+        <v>9.731782496608512</v>
       </c>
       <c r="M18">
-        <v>1.2439278911940529E-3</v>
+        <v>0.001243927891194053</v>
       </c>
       <c r="N18">
-        <v>0.98204791901530941</v>
+        <v>0.9820479190153094</v>
       </c>
       <c r="O18">
-        <v>0.92988073046224473</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.9298807304622447</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15">
       <c r="A19" s="2">
         <v>44351</v>
       </c>
       <c r="B19">
-        <v>1.2144245089022209E-2</v>
+        <v>0.01214424508902221</v>
       </c>
       <c r="C19">
-        <v>2.3023056824755519E-3</v>
+        <v>0.002302305682475552</v>
       </c>
       <c r="D19">
-        <v>3.3459144230440769E-3</v>
+        <v>0.003345914423044077</v>
       </c>
       <c r="E19">
-        <v>0.14273332286762741</v>
+        <v>0.1427333228676274</v>
       </c>
       <c r="F19">
-        <v>0.89286128412700261</v>
+        <v>0.8928612841270026</v>
       </c>
       <c r="G19">
-        <v>4.3207057687729344E-3</v>
+        <v>0.004320705768772934</v>
       </c>
       <c r="H19">
         <v>17</v>
@@ -1319,45 +1298,45 @@
         <v>1</v>
       </c>
       <c r="J19">
-        <v>9.7792270716977274</v>
+        <v>9.779227071697727</v>
       </c>
       <c r="K19">
-        <v>0.95174111535775452</v>
+        <v>0.9517411153577545</v>
       </c>
       <c r="L19">
-        <v>9.2999547699519898</v>
+        <v>9.29995476995199</v>
       </c>
       <c r="M19">
-        <v>2.9559360410858632E-3</v>
+        <v>0.002955936041085863</v>
       </c>
       <c r="N19">
-        <v>0.95716405862004716</v>
+        <v>0.9571640586200472</v>
       </c>
       <c r="O19">
-        <v>0.94238593339308008</v>
-      </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.9423859333930801</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15">
       <c r="A20" s="2">
         <v>44379</v>
       </c>
       <c r="B20">
-        <v>1.4616494030416E-2</v>
+        <v>0.014616494030416</v>
       </c>
       <c r="C20">
-        <v>4.698920320430792E-4</v>
+        <v>0.0004698920320430792</v>
       </c>
       <c r="D20">
-        <v>5.0504265263355119E-3</v>
+        <v>0.005050426526335512</v>
       </c>
       <c r="E20">
-        <v>-0.31535115563097388</v>
+        <v>-0.3153511556309739</v>
       </c>
       <c r="F20">
         <v>0.5291489486109584</v>
       </c>
       <c r="G20">
-        <v>5.9630886640598124E-3</v>
+        <v>0.005963088664059812</v>
       </c>
       <c r="H20">
         <v>22</v>
@@ -1366,45 +1345,45 @@
         <v>3</v>
       </c>
       <c r="J20">
-        <v>10.299885551547129</v>
+        <v>10.29988555154713</v>
       </c>
       <c r="K20">
         <v>1</v>
       </c>
       <c r="L20">
-        <v>8.3461862269119411</v>
+        <v>8.346186226911941</v>
       </c>
       <c r="M20">
-        <v>9.5603676563617585E-3</v>
+        <v>0.009560367656361759</v>
       </c>
       <c r="N20">
-        <v>0.96111169849136258</v>
+        <v>0.9611116984913626</v>
       </c>
       <c r="O20">
-        <v>0.95403323797264394</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.9540332379726439</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15">
       <c r="A21" s="2">
         <v>44414</v>
       </c>
       <c r="B21">
-        <v>1.2987418176994151E-2</v>
+        <v>0.01298741817699415</v>
       </c>
       <c r="C21">
-        <v>-1.431435735320347E-4</v>
+        <v>-0.0001431435735320347</v>
       </c>
       <c r="D21">
-        <v>5.0247012360710927E-3</v>
+        <v>0.005024701236071093</v>
       </c>
       <c r="E21">
-        <v>0.14616314245458889</v>
+        <v>0.1461631424545889</v>
       </c>
       <c r="F21">
-        <v>-0.55541830072337106</v>
+        <v>-0.5554183007233711</v>
       </c>
       <c r="G21">
-        <v>5.3087808739687064E-3</v>
+        <v>0.005308780873968706</v>
       </c>
       <c r="H21">
         <v>19</v>
@@ -1416,42 +1395,42 @@
         <v>10.70110450049223</v>
       </c>
       <c r="K21">
-        <v>0.92181712916856118</v>
+        <v>0.9218171291685612</v>
       </c>
       <c r="L21">
-        <v>7.0831049993621624</v>
+        <v>7.083104999362162</v>
       </c>
       <c r="M21">
-        <v>2.1717609983530669E-2</v>
+        <v>0.02171760998353067</v>
       </c>
       <c r="N21">
-        <v>0.97134481203543643</v>
+        <v>0.9713448120354364</v>
       </c>
       <c r="O21">
-        <v>0.95986868876059861</v>
-      </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.9598686887605986</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15">
       <c r="A22" s="2">
         <v>44442</v>
       </c>
       <c r="B22">
-        <v>1.018453459200962E-2</v>
+        <v>0.01018453459200962</v>
       </c>
       <c r="C22">
-        <v>1.6697933516467631E-3</v>
+        <v>0.001669793351646763</v>
       </c>
       <c r="D22">
-        <v>2.771501412460158E-3</v>
+        <v>0.002771501412460158</v>
       </c>
       <c r="E22">
-        <v>0.33840990188366332</v>
+        <v>0.3384099018836633</v>
       </c>
       <c r="F22">
-        <v>-0.27450763087466817</v>
+        <v>-0.2745076308746682</v>
       </c>
       <c r="G22">
-        <v>6.2207577400391007E-3</v>
+        <v>0.006220757740039101</v>
       </c>
       <c r="H22">
         <v>13</v>
@@ -1460,45 +1439,45 @@
         <v>3</v>
       </c>
       <c r="J22">
-        <v>9.3247518780377021</v>
+        <v>9.324751878037702</v>
       </c>
       <c r="K22">
-        <v>0.75897250666301741</v>
+        <v>0.7589725066630174</v>
       </c>
       <c r="L22">
-        <v>7.2466787436369726</v>
+        <v>7.246678743636973</v>
       </c>
       <c r="M22">
-        <v>1.9394545949518369E-2</v>
+        <v>0.01939454594951837</v>
       </c>
       <c r="N22">
-        <v>0.86705951063401532</v>
+        <v>0.8670595106340153</v>
       </c>
       <c r="O22">
-        <v>0.90689529626094922</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.9068952962609492</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15">
       <c r="A23" s="2">
         <v>44470</v>
       </c>
       <c r="B23">
-        <v>1.1371860278207951E-2</v>
+        <v>0.01137186027820795</v>
       </c>
       <c r="C23">
-        <v>6.5089034789957438E-4</v>
+        <v>0.0006508903478995744</v>
       </c>
       <c r="D23">
-        <v>2.615728784523672E-3</v>
+        <v>0.002615728784523672</v>
       </c>
       <c r="E23">
-        <v>-0.24711858144450149</v>
+        <v>-0.2471185814445015</v>
       </c>
       <c r="F23">
-        <v>-0.56730883955769595</v>
+        <v>-0.567308839557696</v>
       </c>
       <c r="G23">
-        <v>8.7687938747629483E-3</v>
+        <v>0.008768793874762948</v>
       </c>
       <c r="H23">
         <v>16</v>
@@ -1507,45 +1486,45 @@
         <v>9</v>
       </c>
       <c r="J23">
-        <v>8.9587286194040843</v>
+        <v>8.958728619404084</v>
       </c>
       <c r="K23">
-        <v>0.71994332245579651</v>
+        <v>0.7199433224557965</v>
       </c>
       <c r="L23">
-        <v>7.2250056458821028</v>
+        <v>7.225005645882103</v>
       </c>
       <c r="M23">
-        <v>1.3442519145488449E-2</v>
+        <v>0.01344251914548845</v>
       </c>
       <c r="N23">
-        <v>0.73206397652229516</v>
+        <v>0.7320639765222952</v>
       </c>
       <c r="O23">
-        <v>0.82342877523498625</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.8234287752349863</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15">
       <c r="A24" s="2">
         <v>44504</v>
       </c>
       <c r="B24">
-        <v>1.2201682254054529E-2</v>
+        <v>0.01220168225405453</v>
       </c>
       <c r="C24">
-        <v>1.7638757694286771E-3</v>
+        <v>0.001763875769428677</v>
       </c>
       <c r="D24">
-        <v>3.2417674362403238E-3</v>
+        <v>0.003241767436240324</v>
       </c>
       <c r="E24">
-        <v>5.843877591412551E-2</v>
+        <v>0.05843877591412551</v>
       </c>
       <c r="F24">
-        <v>-0.27826196171099399</v>
+        <v>-0.278261961710994</v>
       </c>
       <c r="G24">
-        <v>1.0892415639687561E-2</v>
+        <v>0.01089241563968756</v>
       </c>
       <c r="H24">
         <v>18</v>
@@ -1554,45 +1533,45 @@
         <v>15</v>
       </c>
       <c r="J24">
-        <v>9.3678894140140638</v>
+        <v>9.367889414014064</v>
       </c>
       <c r="K24">
-        <v>0.76357227675454675</v>
+        <v>0.7635722767545468</v>
       </c>
       <c r="L24">
-        <v>8.5173485737947061</v>
+        <v>8.517348573794706</v>
       </c>
       <c r="M24">
-        <v>5.2879294124201174E-3</v>
+        <v>0.005287929412420117</v>
       </c>
       <c r="N24">
-        <v>0.71815115678231689</v>
+        <v>0.7181511567823169</v>
       </c>
       <c r="O24">
-        <v>0.76575246859325885</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.7657524685932589</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15">
       <c r="A25" s="2">
         <v>44533</v>
       </c>
       <c r="B25">
-        <v>1.100813377373416E-2</v>
+        <v>0.01100813377373416</v>
       </c>
       <c r="C25">
-        <v>2.1781028346666551E-3</v>
+        <v>0.002178102834666655</v>
       </c>
       <c r="D25">
-        <v>3.0617911787688E-3</v>
+        <v>0.0030617911787688</v>
       </c>
       <c r="E25">
-        <v>-7.3906182596531714E-2</v>
+        <v>-0.07390618259653171</v>
       </c>
       <c r="F25">
-        <v>-0.71161833259857832</v>
+        <v>-0.7116183325985783</v>
       </c>
       <c r="G25">
-        <v>1.0179225254487591E-2</v>
+        <v>0.01017922525448759</v>
       </c>
       <c r="H25">
         <v>16</v>
@@ -1601,45 +1580,45 @@
         <v>13</v>
       </c>
       <c r="J25">
-        <v>9.7756520535739035</v>
+        <v>9.775652053573904</v>
       </c>
       <c r="K25">
-        <v>0.80705214530610736</v>
+        <v>0.8070521453061074</v>
       </c>
       <c r="L25">
-        <v>8.8615202108558897</v>
+        <v>8.86152021085589</v>
       </c>
       <c r="M25">
-        <v>6.1360299147084386E-3</v>
+        <v>0.006136029914708439</v>
       </c>
       <c r="N25">
-        <v>0.79682911567120374</v>
+        <v>0.7968291156712037</v>
       </c>
       <c r="O25">
-        <v>0.78181892916587126</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.7818189291658713</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15">
       <c r="A26" s="2">
         <v>44568</v>
       </c>
       <c r="B26">
-        <v>1.6170075088997649E-2</v>
+        <v>0.01617007508899765</v>
       </c>
       <c r="C26">
-        <v>4.4248651710167338E-3</v>
+        <v>0.004424865171016734</v>
       </c>
       <c r="D26">
-        <v>9.0580318908324454E-3</v>
+        <v>0.009058031890832445</v>
       </c>
       <c r="E26">
-        <v>0.32518249957080969</v>
+        <v>0.3251824995708097</v>
       </c>
       <c r="F26">
         <v>1.873398923649227</v>
       </c>
       <c r="G26">
-        <v>1.104761601527997E-2</v>
+        <v>0.01104761601527997</v>
       </c>
       <c r="H26">
         <v>24</v>
@@ -1648,45 +1627,45 @@
         <v>16</v>
       </c>
       <c r="J26">
-        <v>10.967525614303041</v>
+        <v>10.96752561430304</v>
       </c>
       <c r="K26">
-        <v>0.93414202731816087</v>
+        <v>0.9341420273181609</v>
       </c>
       <c r="L26">
-        <v>8.3872396702223924</v>
+        <v>8.387239670222392</v>
       </c>
       <c r="M26">
-        <v>1.117613439750367E-2</v>
+        <v>0.01117613439750367</v>
       </c>
       <c r="N26">
-        <v>0.90664756852294426</v>
+        <v>0.9066475685229443</v>
       </c>
       <c r="O26">
-        <v>0.84823312920742844</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.8482331292074284</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15">
       <c r="A27" s="2">
         <v>44596</v>
       </c>
       <c r="B27">
-        <v>1.211877793672037E-2</v>
+        <v>0.01211877793672037</v>
       </c>
       <c r="C27">
-        <v>8.0717417421833867E-4</v>
+        <v>0.0008071741742183387</v>
       </c>
       <c r="D27">
-        <v>3.192573748226837E-3</v>
+        <v>0.003192573748226837</v>
       </c>
       <c r="E27">
         <v>-0.2231594050891785</v>
       </c>
       <c r="F27">
-        <v>-0.32323963253117499</v>
+        <v>-0.323239632531175</v>
       </c>
       <c r="G27">
-        <v>1.8023852664527631E-2</v>
+        <v>0.01802385266452763</v>
       </c>
       <c r="H27">
         <v>18</v>
@@ -1701,39 +1680,39 @@
         <v>0.91740743903249</v>
       </c>
       <c r="L27">
-        <v>8.3877241148398358</v>
+        <v>8.387724114839836</v>
       </c>
       <c r="M27">
-        <v>1.409758676106259E-2</v>
+        <v>0.01409758676106259</v>
       </c>
       <c r="N27">
-        <v>0.91753778673625874</v>
+        <v>0.9175377867362587</v>
       </c>
       <c r="O27">
-        <v>0.88016972113498493</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.8801697211349849</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15">
       <c r="A28" s="2">
         <v>44624</v>
       </c>
       <c r="B28">
-        <v>1.5287896712606041E-2</v>
+        <v>0.01528789671260604</v>
       </c>
       <c r="C28">
-        <v>5.4080846605869878E-5</v>
+        <v>5.408084660586988E-05</v>
       </c>
       <c r="D28">
-        <v>5.9762233497245376E-3</v>
+        <v>0.005976223349724538</v>
       </c>
       <c r="E28">
-        <v>-9.7541976634113237E-2</v>
+        <v>-0.09754197663411324</v>
       </c>
       <c r="F28">
-        <v>-0.39218106326529689</v>
+        <v>-0.3921810632652969</v>
       </c>
       <c r="G28">
-        <v>1.03713455925967E-2</v>
+        <v>0.0103713455925967</v>
       </c>
       <c r="H28">
         <v>23</v>
@@ -1742,45 +1721,45 @@
         <v>14</v>
       </c>
       <c r="J28">
-        <v>11.701019717001349</v>
+        <v>11.70101971700135</v>
       </c>
       <c r="K28">
         <v>1</v>
       </c>
       <c r="L28">
-        <v>9.3064173471285052</v>
+        <v>9.306417347128505</v>
       </c>
       <c r="M28">
-        <v>9.9552953820262798E-3</v>
+        <v>0.00995529538202628</v>
       </c>
       <c r="N28">
-        <v>0.93092143018741458</v>
+        <v>0.9309214301874146</v>
       </c>
       <c r="O28">
-        <v>0.90618395571044108</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.9061839557104411</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15">
       <c r="A29" s="2">
         <v>44652</v>
       </c>
       <c r="B29">
-        <v>1.4315126092353459E-2</v>
+        <v>0.01431512609235346</v>
       </c>
       <c r="C29">
-        <v>-3.9388984092142507E-4</v>
+        <v>-0.0003938898409214251</v>
       </c>
       <c r="D29">
-        <v>5.569712891954349E-3</v>
+        <v>0.005569712891954349</v>
       </c>
       <c r="E29">
-        <v>-8.8682247406075998E-2</v>
+        <v>-0.088682247406076</v>
       </c>
       <c r="F29">
-        <v>-4.1987903022524017E-2</v>
+        <v>-0.04198790302252402</v>
       </c>
       <c r="G29">
-        <v>1.0695339933338989E-2</v>
+        <v>0.01069533993333899</v>
       </c>
       <c r="H29">
         <v>22</v>
@@ -1792,42 +1771,42 @@
         <v>11.49644165166276</v>
       </c>
       <c r="K29">
-        <v>0.95753936229405423</v>
+        <v>0.9575393622940542</v>
       </c>
       <c r="L29">
         <v>12.26131900452658</v>
       </c>
       <c r="M29">
-        <v>-2.9278156745804222E-3</v>
+        <v>-0.002927815674580422</v>
       </c>
       <c r="N29">
-        <v>0.97590483957975083</v>
+        <v>0.9759048395797508</v>
       </c>
       <c r="O29">
-        <v>0.93778354236786265</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.9377835423678627</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15">
       <c r="A30" s="2">
         <v>44687</v>
       </c>
       <c r="B30">
-        <v>1.4101889049837E-2</v>
+        <v>0.014101889049837</v>
       </c>
       <c r="C30">
-        <v>1.623012507228256E-3</v>
+        <v>0.001623012507228256</v>
       </c>
       <c r="D30">
-        <v>4.3441987520018172E-3</v>
+        <v>0.004344198752001817</v>
       </c>
       <c r="E30">
-        <v>-0.49553317777505451</v>
+        <v>-0.4955331777750545</v>
       </c>
       <c r="F30">
         <v>-0.2035430000757579</v>
       </c>
       <c r="G30">
-        <v>1.355073589087105E-2</v>
+        <v>0.01355073589087105</v>
       </c>
       <c r="H30">
         <v>21</v>
@@ -1845,36 +1824,36 @@
         <v>11.50956411572508</v>
       </c>
       <c r="M30">
-        <v>1.820770566585224E-3</v>
+        <v>0.001820770566585224</v>
       </c>
       <c r="N30">
-        <v>0.99939217317186935</v>
+        <v>0.9993921731718693</v>
       </c>
       <c r="O30">
-        <v>0.97032969842678951</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.9703296984267895</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15">
       <c r="A31" s="2">
         <v>44715</v>
       </c>
       <c r="B31">
-        <v>1.961813468762208E-2</v>
+        <v>0.01961813468762208</v>
       </c>
       <c r="C31">
-        <v>-2.5977893211009918E-3</v>
+        <v>-0.002597789321100992</v>
       </c>
       <c r="D31">
-        <v>9.371096650009781E-3</v>
+        <v>0.009371096650009781</v>
       </c>
       <c r="E31">
-        <v>-0.49122311757354242</v>
+        <v>-0.4912231175735424</v>
       </c>
       <c r="F31">
-        <v>0.59180787155763492</v>
+        <v>0.5918078715576349</v>
       </c>
       <c r="G31">
-        <v>1.134301994288088E-2</v>
+        <v>0.01134301994288088</v>
       </c>
       <c r="H31">
         <v>27</v>
@@ -1883,7 +1862,7 @@
         <v>16</v>
       </c>
       <c r="J31">
-        <v>13.482753539589821</v>
+        <v>13.48275353958982</v>
       </c>
       <c r="K31">
         <v>1</v>
@@ -1892,36 +1871,36 @@
         <v>10.50046581577514</v>
       </c>
       <c r="M31">
-        <v>9.2589530945610087E-3</v>
+        <v>0.009258953094561009</v>
       </c>
       <c r="N31">
-        <v>0.98847844151405984</v>
+        <v>0.9884784415140598</v>
       </c>
       <c r="O31">
-        <v>0.97909195215695566</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.9790919521569557</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15">
       <c r="A32" s="2">
         <v>44743</v>
       </c>
       <c r="B32">
-        <v>1.2573438099853569E-2</v>
+        <v>0.01257343809985357</v>
       </c>
       <c r="C32">
-        <v>-4.5613937060039092E-4</v>
+        <v>-0.0004561393706003909</v>
       </c>
       <c r="D32">
-        <v>4.3068255021570644E-3</v>
+        <v>0.004306825502157064</v>
       </c>
       <c r="E32">
-        <v>-0.12568549995242431</v>
+        <v>-0.1256854999524243</v>
       </c>
       <c r="F32">
-        <v>-0.56643564848338812</v>
+        <v>-0.5664356484833881</v>
       </c>
       <c r="G32">
-        <v>7.9631893060199983E-3</v>
+        <v>0.007963189306019998</v>
       </c>
       <c r="H32">
         <v>18</v>
@@ -1930,45 +1909,45 @@
         <v>7</v>
       </c>
       <c r="J32">
-        <v>12.517305325664969</v>
+        <v>12.51730532566497</v>
       </c>
       <c r="K32">
-        <v>0.87107815522795207</v>
+        <v>0.8710781552279521</v>
       </c>
       <c r="L32">
-        <v>11.011789416153119</v>
+        <v>11.01178941615312</v>
       </c>
       <c r="M32">
-        <v>7.1192027196802761E-3</v>
+        <v>0.007119202719680276</v>
       </c>
       <c r="N32">
         <v>0.9363047479147486</v>
       </c>
       <c r="O32">
-        <v>0.95485095793448826</v>
-      </c>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.9548509579344883</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15">
       <c r="A33" s="2">
         <v>44778</v>
       </c>
       <c r="B33">
-        <v>1.314220954616074E-2</v>
+        <v>0.01314220954616074</v>
       </c>
       <c r="C33">
-        <v>-2.4385602103209301E-4</v>
+        <v>-0.000243856021032093</v>
       </c>
       <c r="D33">
-        <v>3.8930644984468358E-3</v>
+        <v>0.003893064498446836</v>
       </c>
       <c r="E33">
-        <v>-5.2796855852304203E-2</v>
+        <v>-0.0527968558523042</v>
       </c>
       <c r="F33">
-        <v>-0.88629294609261733</v>
+        <v>-0.8862929460926173</v>
       </c>
       <c r="G33">
-        <v>1.00357538692675E-2</v>
+        <v>0.0100357538692675</v>
       </c>
       <c r="H33">
         <v>20</v>
@@ -1977,45 +1956,45 @@
         <v>13</v>
       </c>
       <c r="J33">
-        <v>12.547608642401199</v>
+        <v>12.5476086424012</v>
       </c>
       <c r="K33">
-        <v>0.87367439232731281</v>
+        <v>0.8736743923273128</v>
       </c>
       <c r="L33">
-        <v>10.776967438232401</v>
+        <v>10.7769674382324</v>
       </c>
       <c r="M33">
-        <v>7.6059444401072153E-3</v>
+        <v>0.007605944440107215</v>
       </c>
       <c r="N33">
-        <v>0.86689943881129716</v>
+        <v>0.8668994388112972</v>
       </c>
       <c r="O33">
         <v>0.9076497101021489</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:15">
       <c r="A34" s="2">
         <v>44806</v>
       </c>
       <c r="B34">
-        <v>1.189374365782522E-2</v>
+        <v>0.01189374365782522</v>
       </c>
       <c r="C34">
-        <v>3.2624278916141192E-5</v>
+        <v>3.262427891614119E-05</v>
       </c>
       <c r="D34">
-        <v>3.3596273542398779E-3</v>
+        <v>0.003359627354239878</v>
       </c>
       <c r="E34">
-        <v>2.4628499378520671E-2</v>
+        <v>0.02462849937852067</v>
       </c>
       <c r="F34">
-        <v>-0.53392677576772885</v>
+        <v>-0.5339267757677288</v>
       </c>
       <c r="G34">
-        <v>9.8635236208874794E-3</v>
+        <v>0.009863523620887479</v>
       </c>
       <c r="H34">
         <v>17</v>
@@ -2024,45 +2003,45 @@
         <v>12</v>
       </c>
       <c r="J34">
-        <v>11.836505491081541</v>
+        <v>11.83650549108154</v>
       </c>
       <c r="K34">
-        <v>0.81275061956018246</v>
+        <v>0.8127506195601825</v>
       </c>
       <c r="L34">
-        <v>9.9759594291605662</v>
+        <v>9.975959429160566</v>
       </c>
       <c r="M34">
-        <v>1.0059429413692551E-2</v>
+        <v>0.01005942941369255</v>
       </c>
       <c r="N34">
-        <v>0.82105554082850729</v>
+        <v>0.8210555408285073</v>
       </c>
       <c r="O34">
         <v>0.8659748637358925</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:15">
       <c r="A35" s="2">
         <v>44841</v>
       </c>
       <c r="B35">
-        <v>1.1906960590838371E-2</v>
+        <v>0.01190696059083837</v>
       </c>
       <c r="C35">
-        <v>3.9111235196303488E-4</v>
+        <v>0.0003911123519630349</v>
       </c>
       <c r="D35">
-        <v>3.175838181172608E-3</v>
+        <v>0.003175838181172608</v>
       </c>
       <c r="E35">
-        <v>8.008899907397754E-2</v>
+        <v>0.08008899907397754</v>
       </c>
       <c r="F35">
-        <v>-0.24364395154327231</v>
+        <v>-0.2436439515432723</v>
       </c>
       <c r="G35">
-        <v>6.7957165077963313E-3</v>
+        <v>0.006795716507796331</v>
       </c>
       <c r="H35">
         <v>17</v>
@@ -2074,42 +2053,42 @@
         <v>12.02119770080113</v>
       </c>
       <c r="K35">
-        <v>0.82857412729732827</v>
+        <v>0.8285741272973283</v>
       </c>
       <c r="L35">
         <v>10.78670342409159</v>
       </c>
       <c r="M35">
-        <v>6.3739620755288301E-3</v>
+        <v>0.00637396207552883</v>
       </c>
       <c r="N35">
-        <v>0.81267535198249308</v>
+        <v>0.8126753519824931</v>
       </c>
       <c r="O35">
-        <v>0.83523200670385611</v>
-      </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.8352320067038561</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15">
       <c r="A36" s="2">
         <v>44869</v>
       </c>
       <c r="B36">
-        <v>9.5944445040354164E-3</v>
+        <v>0.009594444504035416</v>
       </c>
       <c r="C36">
-        <v>2.8149054767362628E-3</v>
+        <v>0.002814905476736263</v>
       </c>
       <c r="D36">
-        <v>2.375616237963001E-3</v>
+        <v>0.002375616237963001</v>
       </c>
       <c r="E36">
-        <v>-0.26267435092592328</v>
+        <v>-0.2626743509259233</v>
       </c>
       <c r="F36">
         <v>-0.4967028217928548</v>
       </c>
       <c r="G36">
-        <v>6.5050324883238787E-3</v>
+        <v>0.006505032488323879</v>
       </c>
       <c r="H36">
         <v>12</v>
@@ -2121,42 +2100,42 @@
         <v>11.76313457058292</v>
       </c>
       <c r="K36">
-        <v>0.80646456488600793</v>
+        <v>0.8064645648860079</v>
       </c>
       <c r="L36">
         <v>10.9288488827174</v>
       </c>
       <c r="M36">
-        <v>6.1303727212716919E-3</v>
+        <v>0.006130372721271692</v>
       </c>
       <c r="N36">
-        <v>0.81353938822146943</v>
+        <v>0.8135393882214694</v>
       </c>
       <c r="O36">
-        <v>0.82433996514630348</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.8243399651463035</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15">
       <c r="A37" s="2">
         <v>44897</v>
       </c>
       <c r="B37">
-        <v>1.400626653951385E-2</v>
+        <v>0.01400626653951385</v>
       </c>
       <c r="C37">
-        <v>1.4738696615584201E-3</v>
+        <v>0.00147386966155842</v>
       </c>
       <c r="D37">
-        <v>4.0869127464148039E-3</v>
+        <v>0.004086912746414804</v>
       </c>
       <c r="E37">
-        <v>0.14316425913639211</v>
+        <v>0.1431642591363921</v>
       </c>
       <c r="F37">
         <v>-0.2430681649332877</v>
       </c>
       <c r="G37">
-        <v>7.4738317634562247E-3</v>
+        <v>0.007473831763456225</v>
       </c>
       <c r="H37">
         <v>21</v>
@@ -2165,45 +2144,45 @@
         <v>6</v>
       </c>
       <c r="J37">
-        <v>12.483465084283029</v>
+        <v>12.48346508428303</v>
       </c>
       <c r="K37">
-        <v>0.86817889205844956</v>
+        <v>0.8681788920584496</v>
       </c>
       <c r="L37">
-        <v>10.979233217776301</v>
+        <v>10.9792332177763</v>
       </c>
       <c r="M37">
-        <v>6.1142560091121219E-3</v>
+        <v>0.006114256009112122</v>
       </c>
       <c r="N37">
-        <v>0.84507930999457403</v>
+        <v>0.845079309994574</v>
       </c>
       <c r="O37">
-        <v>0.83671952441748665</v>
-      </c>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.8367195244174866</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15">
       <c r="A38" s="2">
         <v>44932</v>
       </c>
       <c r="B38">
-        <v>1.3988701908054801E-2</v>
+        <v>0.0139887019080548</v>
       </c>
       <c r="C38">
-        <v>-7.0910067550102192E-4</v>
+        <v>-0.0007091006755010219</v>
       </c>
       <c r="D38">
-        <v>4.0082242327292121E-3</v>
+        <v>0.004008224232729212</v>
       </c>
       <c r="E38">
-        <v>0.33109557276398383</v>
+        <v>0.3310955727639838</v>
       </c>
       <c r="F38">
-        <v>0.34141543054101048</v>
+        <v>0.3414154305410105</v>
       </c>
       <c r="G38">
-        <v>7.278654461335729E-3</v>
+        <v>0.007278654461335729</v>
       </c>
       <c r="H38">
         <v>21</v>
@@ -2212,45 +2191,45 @@
         <v>5</v>
       </c>
       <c r="J38">
-        <v>12.560342598225819</v>
+        <v>12.56034259822582</v>
       </c>
       <c r="K38">
-        <v>0.87476537417663525</v>
+        <v>0.8747653741766352</v>
       </c>
       <c r="L38">
         <v>10.5469735706083</v>
       </c>
       <c r="M38">
-        <v>8.3193087701759448E-3</v>
+        <v>0.008319308770175945</v>
       </c>
       <c r="N38">
-        <v>0.85364563947912109</v>
+        <v>0.8536456394791211</v>
       </c>
       <c r="O38">
-        <v>0.84593116204548768</v>
-      </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.8459311620454877</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15">
       <c r="A39" s="2">
         <v>44960</v>
       </c>
       <c r="B39">
-        <v>1.1950507090984479E-2</v>
+        <v>0.01195050709098448</v>
       </c>
       <c r="C39">
-        <v>2.0359245800991368E-3</v>
+        <v>0.002035924580099137</v>
       </c>
       <c r="D39">
-        <v>3.0085005262177091E-3</v>
+        <v>0.003008500526217709</v>
       </c>
       <c r="E39">
-        <v>-3.3614648674700667E-2</v>
+        <v>-0.03361464867470067</v>
       </c>
       <c r="F39">
-        <v>0.54650282598782984</v>
+        <v>0.5465028259878298</v>
       </c>
       <c r="G39">
-        <v>7.1796611837523791E-3</v>
+        <v>0.007179661183752379</v>
       </c>
       <c r="H39">
         <v>18</v>
@@ -2259,16 +2238,16 @@
         <v>5</v>
       </c>
       <c r="J39">
-        <v>12.141013212041999</v>
+        <v>12.141013212042</v>
       </c>
       <c r="K39">
-        <v>0.83883932295462482</v>
+        <v>0.8388393229546248</v>
       </c>
       <c r="L39">
         <v>10.19294850310447</v>
       </c>
       <c r="M39">
-        <v>9.7162824881730815E-3</v>
+        <v>0.009716282488173082</v>
       </c>
       <c r="N39">
         <v>0.8242915310778558</v>
@@ -2277,27 +2256,27 @@
         <v>0.8359588974196086</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:15">
       <c r="A40" s="2">
         <v>44988</v>
       </c>
       <c r="B40">
-        <v>1.038039164379939E-2</v>
+        <v>0.01038039164379939</v>
       </c>
       <c r="C40">
-        <v>5.9028822143684858E-4</v>
+        <v>0.0005902882214368486</v>
       </c>
       <c r="D40">
-        <v>2.2836366538595428E-3</v>
+        <v>0.002283636653859543</v>
       </c>
       <c r="E40">
-        <v>-0.12198806494529089</v>
+        <v>-0.1219880649452909</v>
       </c>
       <c r="F40">
-        <v>0.84663036343957232</v>
+        <v>0.8466303634395723</v>
       </c>
       <c r="G40">
-        <v>7.741536223600967E-3</v>
+        <v>0.007741536223600967</v>
       </c>
       <c r="H40">
         <v>14</v>
@@ -2309,42 +2288,42 @@
         <v>10.82999474672356</v>
       </c>
       <c r="K40">
-        <v>0.72651779698986707</v>
+        <v>0.7265177969898671</v>
       </c>
       <c r="L40">
-        <v>8.6826995899700936</v>
+        <v>8.682699589970094</v>
       </c>
       <c r="M40">
-        <v>1.5784791639892531E-2</v>
+        <v>0.01578479163989253</v>
       </c>
       <c r="N40">
-        <v>0.72438512556157808</v>
+        <v>0.7243851255615781</v>
       </c>
       <c r="O40">
-        <v>0.78083251877187132</v>
-      </c>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.7808325187718713</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15">
       <c r="A41" s="2">
         <v>45022</v>
       </c>
       <c r="B41">
-        <v>1.01917896021158E-2</v>
+        <v>0.0101917896021158</v>
       </c>
       <c r="C41">
-        <v>1.270165010610131E-3</v>
+        <v>0.001270165010610131</v>
       </c>
       <c r="D41">
-        <v>2.395833979080613E-3</v>
+        <v>0.002395833979080613</v>
       </c>
       <c r="E41">
-        <v>0.36764850999452781</v>
+        <v>0.3676485099945278</v>
       </c>
       <c r="F41">
-        <v>9.7878841969948671E-2</v>
+        <v>0.09787884196994867</v>
       </c>
       <c r="G41">
-        <v>5.3371899753572134E-3</v>
+        <v>0.005337189975357213</v>
       </c>
       <c r="H41">
         <v>14</v>
@@ -2356,42 +2335,42 @@
         <v>10.5179083054421</v>
       </c>
       <c r="K41">
-        <v>0.65784628767506248</v>
+        <v>0.6578462876750625</v>
       </c>
       <c r="L41">
-        <v>8.9073562067994381</v>
+        <v>8.907356206799438</v>
       </c>
       <c r="M41">
-        <v>1.187156298766213E-2</v>
+        <v>0.01187156298766213</v>
       </c>
       <c r="N41">
-        <v>0.76469045984434292</v>
+        <v>0.7646904598443429</v>
       </c>
       <c r="O41">
-        <v>0.76511899872332989</v>
-      </c>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.7651189987233299</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15">
       <c r="A42" s="2">
         <v>45051</v>
       </c>
       <c r="B42">
-        <v>1.1237445892589929E-2</v>
+        <v>0.01123744589258993</v>
       </c>
       <c r="C42">
-        <v>1.359828527878064E-3</v>
+        <v>0.001359828527878064</v>
       </c>
       <c r="D42">
-        <v>2.780460531101806E-3</v>
+        <v>0.002780460531101806</v>
       </c>
       <c r="E42">
         <v>0.111086054541347</v>
       </c>
       <c r="F42">
-        <v>-0.64649213714618159</v>
+        <v>-0.6464921371461816</v>
       </c>
       <c r="G42">
-        <v>4.2492594928200218E-3</v>
+        <v>0.004249259492820022</v>
       </c>
       <c r="H42">
         <v>16</v>
@@ -2403,42 +2382,42 @@
         <v>10.45619213915667</v>
       </c>
       <c r="K42">
-        <v>0.57585057309836796</v>
+        <v>0.575850573098368</v>
       </c>
       <c r="L42">
         <v>8.471668034190122</v>
       </c>
       <c r="M42">
-        <v>1.3154183029407769E-2</v>
+        <v>0.01315418302940777</v>
       </c>
       <c r="N42">
-        <v>0.63606278906602531</v>
+        <v>0.6360627890660253</v>
       </c>
       <c r="O42">
-        <v>0.70030148324874886</v>
-      </c>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.7003014832487489</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15">
       <c r="A43" s="2">
         <v>45079</v>
       </c>
       <c r="B43">
-        <v>1.0736516071105149E-2</v>
+        <v>0.01073651607110515</v>
       </c>
       <c r="C43">
-        <v>-8.0120308256035905E-4</v>
+        <v>-0.0008012030825603591</v>
       </c>
       <c r="D43">
-        <v>2.4597464783437978E-3</v>
+        <v>0.002459746478343798</v>
       </c>
       <c r="E43">
-        <v>6.0594199554696158E-2</v>
+        <v>0.06059419955469616</v>
       </c>
       <c r="F43">
         <v>-0.1860096059785539</v>
       </c>
       <c r="G43">
-        <v>5.2648755466127182E-3</v>
+        <v>0.005264875546612718</v>
       </c>
       <c r="H43">
         <v>15</v>
@@ -2447,45 +2426,45 @@
         <v>2</v>
       </c>
       <c r="J43">
-        <v>9.3783597444920659</v>
+        <v>9.378359744492066</v>
       </c>
       <c r="K43">
-        <v>0.42958249604780863</v>
+        <v>0.4295824960478086</v>
       </c>
       <c r="L43">
-        <v>7.4157384126847514</v>
+        <v>7.415738412684751</v>
       </c>
       <c r="M43">
-        <v>1.565335507540901E-2</v>
+        <v>0.01565335507540901</v>
       </c>
       <c r="N43">
-        <v>0.53569770441464559</v>
+        <v>0.5356977044146456</v>
       </c>
       <c r="O43">
-        <v>0.61412822162250613</v>
-      </c>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.6141282216225061</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15">
       <c r="A44" s="2">
         <v>45114</v>
       </c>
       <c r="B44">
-        <v>1.110714603681006E-2</v>
+        <v>0.01110714603681006</v>
       </c>
       <c r="C44">
-        <v>7.1853412514844678E-4</v>
+        <v>0.0007185341251484468</v>
       </c>
       <c r="D44">
-        <v>2.96679535779166E-3</v>
+        <v>0.00296679535779166</v>
       </c>
       <c r="E44">
         <v>-0.2028576299145336</v>
       </c>
       <c r="F44">
-        <v>-0.20778864042548501</v>
+        <v>-0.207788640425485</v>
       </c>
       <c r="G44">
-        <v>6.0150377960345378E-3</v>
+        <v>0.006015037796034538</v>
       </c>
       <c r="H44">
         <v>16</v>
@@ -2494,45 +2473,45 @@
         <v>3</v>
       </c>
       <c r="J44">
-        <v>8.5646292329569125</v>
+        <v>8.564629232956912</v>
       </c>
       <c r="K44">
-        <v>0.29343944012643669</v>
+        <v>0.2934394401264367</v>
       </c>
       <c r="L44">
         <v>5.332490065354726</v>
       </c>
       <c r="M44">
-        <v>2.9613908368316639E-2</v>
+        <v>0.02961390836831664</v>
       </c>
       <c r="N44">
-        <v>0.42347303349524762</v>
+        <v>0.4234730334952476</v>
       </c>
       <c r="O44">
-        <v>0.49547041004509751</v>
-      </c>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.4954704100450975</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15">
       <c r="A45" s="2">
         <v>45142</v>
       </c>
       <c r="B45">
-        <v>1.060995110861576E-2</v>
+        <v>0.01060995110861576</v>
       </c>
       <c r="C45">
-        <v>3.2691904149726841E-4</v>
+        <v>0.0003269190414972684</v>
       </c>
       <c r="D45">
-        <v>2.332934356695278E-3</v>
+        <v>0.002332934356695278</v>
       </c>
       <c r="E45">
         <v>0.2043035221423094</v>
       </c>
       <c r="F45">
-        <v>-0.20566298345854031</v>
+        <v>-0.2056629834585403</v>
       </c>
       <c r="G45">
-        <v>4.2103905881875261E-3</v>
+        <v>0.004210390588187526</v>
       </c>
       <c r="H45">
         <v>15</v>
@@ -2541,45 +2520,45 @@
         <v>1</v>
       </c>
       <c r="J45">
-        <v>8.1033005777782297</v>
+        <v>8.10330057777823</v>
       </c>
       <c r="K45">
-        <v>0.22614207821505281</v>
+        <v>0.2261420782150528</v>
       </c>
       <c r="L45">
-        <v>5.2071288319399116</v>
+        <v>5.207128831939912</v>
       </c>
       <c r="M45">
-        <v>2.9482856098561092E-2</v>
+        <v>0.02948285609856109</v>
       </c>
       <c r="N45">
-        <v>0.30956689514745911</v>
+        <v>0.3095668951474591</v>
       </c>
       <c r="O45">
-        <v>0.39876645919516568</v>
-      </c>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.3987664591951657</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15">
       <c r="A46" s="2">
         <v>45170</v>
       </c>
       <c r="B46">
-        <v>1.062048173176806E-2</v>
+        <v>0.01062048173176806</v>
       </c>
       <c r="C46">
-        <v>-2.1095328369072522E-3</v>
+        <v>-0.002109532836907252</v>
       </c>
       <c r="D46">
-        <v>2.5814387288340709E-3</v>
+        <v>0.002581438728834071</v>
       </c>
       <c r="E46">
-        <v>-0.36590929843434072</v>
+        <v>-0.3659092984343407</v>
       </c>
       <c r="F46">
-        <v>6.9357681161351672E-2</v>
+        <v>0.06935768116135167</v>
       </c>
       <c r="G46">
-        <v>5.6103668690779592E-3</v>
+        <v>0.005610366869077959</v>
       </c>
       <c r="H46">
         <v>15</v>
@@ -2588,45 +2567,45 @@
         <v>2</v>
       </c>
       <c r="J46">
-        <v>6.9566729599976984</v>
+        <v>6.956672959997698</v>
       </c>
       <c r="K46">
-        <v>9.3502499858121466E-2</v>
+        <v>0.09350249985812147</v>
       </c>
       <c r="L46">
-        <v>3.4547480550125238</v>
+        <v>3.454748055012524</v>
       </c>
       <c r="M46">
-        <v>4.6663453623742433E-2</v>
+        <v>0.04666345362374243</v>
       </c>
       <c r="N46">
-        <v>4.27729346108911E-2</v>
+        <v>0.0427729346108911</v>
       </c>
       <c r="O46">
-        <v>0.22933138264090749</v>
-      </c>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.2293313826409075</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15">
       <c r="A47" s="2">
         <v>45205</v>
       </c>
       <c r="B47">
-        <v>8.8051250500022719E-3</v>
+        <v>0.008805125050002272</v>
       </c>
       <c r="C47">
-        <v>-4.0105124478447593E-4</v>
+        <v>-0.0004010512447844759</v>
       </c>
       <c r="D47">
-        <v>1.7848439938138109E-3</v>
+        <v>0.001784843993813811</v>
       </c>
       <c r="E47">
-        <v>-0.17097844018777969</v>
+        <v>-0.1709784401877797</v>
       </c>
       <c r="F47">
-        <v>-0.48983151330035291</v>
+        <v>-0.4898315133003529</v>
       </c>
       <c r="G47">
-        <v>7.3974225534427602E-3</v>
+        <v>0.00739742255344276</v>
       </c>
       <c r="H47">
         <v>10</v>
@@ -2635,45 +2614,45 @@
         <v>6</v>
       </c>
       <c r="J47">
-        <v>4.8197007386080726</v>
+        <v>4.819700738608073</v>
       </c>
       <c r="K47">
         <v>0</v>
       </c>
       <c r="L47">
-        <v>2.8491346865536702</v>
+        <v>2.84913468655367</v>
       </c>
       <c r="M47">
-        <v>5.256965092833385E-2</v>
+        <v>0.05256965092833385</v>
       </c>
       <c r="N47">
         <v>0.102383245451479</v>
       </c>
       <c r="O47">
-        <v>0.15127610892958551</v>
-      </c>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.1512761089295855</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15">
       <c r="A48" s="2">
         <v>45233</v>
       </c>
       <c r="B48">
-        <v>1.0252644815586029E-2</v>
+        <v>0.01025264481558603</v>
       </c>
       <c r="C48">
-        <v>1.583586721117533E-3</v>
+        <v>0.001583586721117533</v>
       </c>
       <c r="D48">
-        <v>2.3453848531306471E-3</v>
+        <v>0.002345384853130647</v>
       </c>
       <c r="E48">
-        <v>-6.5110819064149256E-2</v>
+        <v>-0.06511081906414926</v>
       </c>
       <c r="F48">
         <v>-0.3250352652700047</v>
       </c>
       <c r="G48">
-        <v>4.3651511842585956E-3</v>
+        <v>0.004365151184258596</v>
       </c>
       <c r="H48">
         <v>14</v>
@@ -2682,45 +2661,45 @@
         <v>1</v>
       </c>
       <c r="J48">
-        <v>5.8257016725619168</v>
+        <v>5.825701672561917</v>
       </c>
       <c r="K48">
-        <v>0.10931962080800969</v>
+        <v>0.1093196208080097</v>
       </c>
       <c r="L48">
-        <v>3.3365505700818709</v>
+        <v>3.336550570081871</v>
       </c>
       <c r="M48">
-        <v>3.9810138652404778E-2</v>
+        <v>0.03981013865240478</v>
       </c>
       <c r="N48">
-        <v>0.33941238162045972</v>
+        <v>0.3394123816204597</v>
       </c>
       <c r="O48">
         <v>0.2245726481737125</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:15">
       <c r="A49" s="2">
         <v>45261</v>
       </c>
       <c r="B49">
-        <v>9.0045143962093864E-3</v>
+        <v>0.009004514396209386</v>
       </c>
       <c r="C49">
-        <v>2.1690995790128059E-3</v>
+        <v>0.002169099579012806</v>
       </c>
       <c r="D49">
-        <v>2.0414274161165572E-3</v>
+        <v>0.002041427416116557</v>
       </c>
       <c r="E49">
-        <v>0.30955416680093678</v>
+        <v>0.3095541668009368</v>
       </c>
       <c r="F49">
-        <v>0.54988278583709216</v>
+        <v>0.5498827858370922</v>
       </c>
       <c r="G49">
-        <v>6.2651650510796349E-3</v>
+        <v>0.006265165051079635</v>
       </c>
       <c r="H49">
         <v>11</v>
@@ -2729,45 +2708,45 @@
         <v>4</v>
       </c>
       <c r="J49">
-        <v>4.8995725940658019</v>
+        <v>4.899572594065802</v>
       </c>
       <c r="K49">
-        <v>8.6794759897028586E-3</v>
+        <v>0.008679475989702859</v>
       </c>
       <c r="L49">
-        <v>2.9585319513347779</v>
+        <v>2.958531951334778</v>
       </c>
       <c r="M49">
-        <v>4.5859526608390641E-2</v>
+        <v>0.04585952660839064</v>
       </c>
       <c r="N49">
-        <v>0.24723992734013439</v>
+        <v>0.2472399273401344</v>
       </c>
       <c r="O49">
         <v>0.2231862798973839</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:15">
       <c r="A50" s="2">
         <v>45296</v>
       </c>
       <c r="B50">
-        <v>1.0349644740779349E-2</v>
+        <v>0.01034964474077935</v>
       </c>
       <c r="C50">
-        <v>6.067070507773172E-4</v>
+        <v>0.0006067070507773172</v>
       </c>
       <c r="D50">
-        <v>2.378543026526334E-3</v>
+        <v>0.002378543026526334</v>
       </c>
       <c r="E50">
-        <v>5.6700101828864542E-2</v>
+        <v>0.05670010182886454</v>
       </c>
       <c r="F50">
-        <v>0.26865570234090641</v>
+        <v>0.2686557023409064</v>
       </c>
       <c r="G50">
-        <v>9.717124662793104E-3</v>
+        <v>0.009717124662793104</v>
       </c>
       <c r="H50">
         <v>14</v>
@@ -2776,45 +2755,45 @@
         <v>13</v>
       </c>
       <c r="J50">
-        <v>5.8994627096806527</v>
+        <v>5.899462709680653</v>
       </c>
       <c r="K50">
         <v>0.1173350493588898</v>
       </c>
       <c r="L50">
-        <v>3.3201236372304499</v>
+        <v>3.32012363723045</v>
       </c>
       <c r="M50">
-        <v>4.1061375588887401E-2</v>
+        <v>0.0410613755888874</v>
       </c>
       <c r="N50">
-        <v>0.16396412042392269</v>
+        <v>0.1639641204239227</v>
       </c>
       <c r="O50">
         <v>0.18329660616926</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:15">
       <c r="A51" s="2">
         <v>45324</v>
       </c>
       <c r="B51">
-        <v>9.2759244529142769E-3</v>
+        <v>0.009275924452914277</v>
       </c>
       <c r="C51">
-        <v>1.3778193515007349E-3</v>
+        <v>0.001377819351500735</v>
       </c>
       <c r="D51">
-        <v>2.027541692072457E-3</v>
+        <v>0.002027541692072457</v>
       </c>
       <c r="E51">
-        <v>0.13567454892226949</v>
+        <v>0.1356745489222695</v>
       </c>
       <c r="F51">
-        <v>0.44953471474113188</v>
+        <v>0.4495347147411319</v>
       </c>
       <c r="G51">
-        <v>6.5493284026386083E-3</v>
+        <v>0.006549328402638608</v>
       </c>
       <c r="H51">
         <v>12</v>
@@ -2823,36 +2802,36 @@
         <v>5</v>
       </c>
       <c r="J51">
-        <v>5.0745865375338681</v>
+        <v>5.074586537533868</v>
       </c>
       <c r="K51">
-        <v>2.7697806182347851E-2</v>
+        <v>0.02769780618234785</v>
       </c>
       <c r="L51">
-        <v>2.9719617073445872</v>
+        <v>2.971961707344587</v>
       </c>
       <c r="M51">
-        <v>4.458523407277741E-2</v>
+        <v>0.04458523407277741</v>
       </c>
       <c r="N51">
-        <v>9.3011201633786872E-2</v>
+        <v>0.09301120163378687</v>
       </c>
       <c r="O51">
-        <v>0.13872593615589121</v>
-      </c>
-    </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.1387259361558912</v>
+      </c>
+    </row>
+    <row r="52" spans="1:15">
       <c r="A52" s="2">
         <v>45353</v>
       </c>
       <c r="B52">
-        <v>1.298438592515838E-2</v>
+        <v>0.01298438592515838</v>
       </c>
       <c r="C52">
-        <v>2.7117772498965382E-3</v>
+        <v>0.002711777249896538</v>
       </c>
       <c r="D52">
-        <v>3.5538598578968151E-3</v>
+        <v>0.003553859857896815</v>
       </c>
       <c r="E52">
         <v>-0.1331323146299829</v>
@@ -2861,7 +2840,7 @@
         <v>0.543910865640715</v>
       </c>
       <c r="G52">
-        <v>6.6645305170528494E-3</v>
+        <v>0.006664530517052849</v>
       </c>
       <c r="H52">
         <v>20</v>
@@ -2870,45 +2849,45 @@
         <v>5</v>
       </c>
       <c r="J52">
-        <v>7.0018741134060187</v>
+        <v>7.001874113406019</v>
       </c>
       <c r="K52">
-        <v>0.23713135626292711</v>
+        <v>0.2371313562629271</v>
       </c>
       <c r="L52">
-        <v>3.1530719018095872</v>
+        <v>3.153071901809587</v>
       </c>
       <c r="M52">
-        <v>3.989003295763021E-2</v>
+        <v>0.03989003295763021</v>
       </c>
       <c r="N52">
-        <v>0.38357695109166429</v>
+        <v>0.3835769510916643</v>
       </c>
       <c r="O52">
         <v>0.2489783934928117</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:15">
       <c r="A53" s="2">
         <v>45387</v>
       </c>
       <c r="B53">
-        <v>1.024167648940367E-2</v>
+        <v>0.01024167648940367</v>
       </c>
       <c r="C53">
-        <v>2.554863032690109E-4</v>
+        <v>0.0002554863032690109</v>
       </c>
       <c r="D53">
-        <v>2.1867285895398568E-3</v>
+        <v>0.002186728589539857</v>
       </c>
       <c r="E53">
         <v>-0.1234385731474428</v>
       </c>
       <c r="F53">
-        <v>0.72955642462851245</v>
+        <v>0.7295564246285124</v>
       </c>
       <c r="G53">
-        <v>6.9039220824454748E-3</v>
+        <v>0.006903922082445475</v>
       </c>
       <c r="H53">
         <v>14</v>
@@ -2917,45 +2896,45 @@
         <v>5</v>
       </c>
       <c r="J53">
-        <v>5.0310269854616081</v>
+        <v>5.031026985461608</v>
       </c>
       <c r="K53">
-        <v>5.8037668430273678E-2</v>
+        <v>0.05803766843027368</v>
       </c>
       <c r="L53">
         <v>2.888770929533746</v>
       </c>
       <c r="M53">
-        <v>3.962807196887097E-2</v>
+        <v>0.03962807196887097</v>
       </c>
       <c r="N53">
-        <v>8.0564376923091485E-2</v>
+        <v>0.08056437692309149</v>
       </c>
       <c r="O53">
-        <v>0.15614543255492419</v>
-      </c>
-    </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.1561454325549242</v>
+      </c>
+    </row>
+    <row r="54" spans="1:15">
       <c r="A54" s="2">
         <v>45415</v>
       </c>
       <c r="B54">
-        <v>9.771918795340161E-3</v>
+        <v>0.009771918795340161</v>
       </c>
       <c r="C54">
-        <v>1.9516773057935461E-3</v>
+        <v>0.001951677305793546</v>
       </c>
       <c r="D54">
-        <v>2.2515438398912789E-3</v>
+        <v>0.002251543839891279</v>
       </c>
       <c r="E54">
-        <v>-0.12949274603124469</v>
+        <v>-0.1294927460312447</v>
       </c>
       <c r="F54">
-        <v>0.13901068033633199</v>
+        <v>0.139010680336332</v>
       </c>
       <c r="G54">
-        <v>9.8868116706273095E-3</v>
+        <v>0.009886811670627309</v>
       </c>
       <c r="H54">
         <v>13</v>
@@ -2964,45 +2943,45 @@
         <v>14</v>
       </c>
       <c r="J54">
-        <v>3.7753267730842399</v>
+        <v>3.77532677308424</v>
       </c>
       <c r="K54">
         <v>0</v>
       </c>
       <c r="L54">
-        <v>1.6462305016194829</v>
+        <v>1.646230501619483</v>
       </c>
       <c r="M54">
-        <v>6.3846062421127212E-2</v>
+        <v>0.06384606242112721</v>
       </c>
       <c r="N54">
-        <v>1.9689416168145471E-2</v>
+        <v>0.01968941616814547</v>
       </c>
       <c r="O54">
-        <v>8.9433688184475363E-2</v>
-      </c>
-    </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.08943368818447536</v>
+      </c>
+    </row>
+    <row r="55" spans="1:15">
       <c r="A55" s="2">
         <v>45450</v>
       </c>
       <c r="B55">
-        <v>1.081135291627505E-2</v>
+        <v>0.01081135291627505</v>
       </c>
       <c r="C55">
-        <v>8.4162611955700779E-5</v>
+        <v>8.416261195570078E-05</v>
       </c>
       <c r="D55">
-        <v>2.5540056292915909E-3</v>
+        <v>0.002554005629291591</v>
       </c>
       <c r="E55">
-        <v>0.14418663764968459</v>
+        <v>0.1441866376496846</v>
       </c>
       <c r="F55">
-        <v>-0.71325518252014286</v>
+        <v>-0.7132551825201429</v>
       </c>
       <c r="G55">
-        <v>4.0961505817649546E-3</v>
+        <v>0.004096150581764955</v>
       </c>
       <c r="H55">
         <v>16</v>
@@ -3011,45 +2990,45 @@
         <v>1</v>
       </c>
       <c r="J55">
-        <v>4.6955478054840656</v>
+        <v>4.695547805484066</v>
       </c>
       <c r="K55">
-        <v>8.9806082671514534E-2</v>
+        <v>0.08980608267151453</v>
       </c>
       <c r="L55">
-        <v>1.4622593464953659</v>
+        <v>1.462259346495366</v>
       </c>
       <c r="M55">
-        <v>7.2914502947432652E-2</v>
+        <v>0.07291450294743265</v>
       </c>
       <c r="N55">
-        <v>0.25728927851435901</v>
+        <v>0.257289278514359</v>
       </c>
       <c r="O55">
-        <v>0.16246304671466599</v>
-      </c>
-    </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.162463046714666</v>
+      </c>
+    </row>
+    <row r="56" spans="1:15">
       <c r="A56" s="2">
         <v>45478</v>
       </c>
       <c r="B56">
-        <v>1.082316985497896E-2</v>
+        <v>0.01082316985497896</v>
       </c>
       <c r="C56">
-        <v>2.744273877016791E-3</v>
+        <v>0.002744273877016791</v>
       </c>
       <c r="D56">
-        <v>2.8659160260348991E-3</v>
+        <v>0.002865916026034899</v>
       </c>
       <c r="E56">
-        <v>0.17505352783055839</v>
+        <v>0.1750535278305584</v>
       </c>
       <c r="F56">
-        <v>0.24735440079802951</v>
+        <v>0.2473544007980295</v>
       </c>
       <c r="G56">
-        <v>9.0619855405483438E-3</v>
+        <v>0.009061985540548344</v>
       </c>
       <c r="H56">
         <v>16</v>
@@ -3058,7 +3037,7 @@
         <v>11</v>
       </c>
       <c r="J56">
-        <v>4.8913356298760151</v>
+        <v>4.891335629876015</v>
       </c>
       <c r="K56">
         <v>0.1143483440635122</v>
@@ -3067,36 +3046,36 @@
         <v>1.568971682328373</v>
       </c>
       <c r="M56">
-        <v>7.1065310986086039E-2</v>
+        <v>0.07106531098608604</v>
       </c>
       <c r="N56">
-        <v>0.11036224110836571</v>
+        <v>0.1103622411083657</v>
       </c>
       <c r="O56">
         <v>0.1347790564778848</v>
       </c>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:15">
       <c r="A57" s="2">
         <v>45506</v>
       </c>
       <c r="B57">
-        <v>1.153693467558818E-2</v>
+        <v>0.01153693467558818</v>
       </c>
       <c r="C57">
-        <v>1.131415350643311E-3</v>
+        <v>0.001131415350643311</v>
       </c>
       <c r="D57">
-        <v>2.8317356224835119E-3</v>
+        <v>0.002831735622483512</v>
       </c>
       <c r="E57">
-        <v>-4.2233646423621631E-2</v>
+        <v>-0.04223364642362163</v>
       </c>
       <c r="F57">
-        <v>-0.26981368350000329</v>
+        <v>-0.2698136835000033</v>
       </c>
       <c r="G57">
-        <v>6.1137811299511484E-3</v>
+        <v>0.006113781129951148</v>
       </c>
       <c r="H57">
         <v>18</v>
@@ -3111,39 +3090,39 @@
         <v>0.2191399180097228</v>
       </c>
       <c r="L57">
-        <v>1.8798169354246359</v>
+        <v>1.879816935424636</v>
       </c>
       <c r="M57">
-        <v>6.4214279817610978E-2</v>
+        <v>0.06421427981761098</v>
       </c>
       <c r="N57">
-        <v>0.14910867323804489</v>
+        <v>0.1491086732380449</v>
       </c>
       <c r="O57">
         <v>0.1448228716615054</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:15">
       <c r="A58" s="2">
         <v>45541</v>
       </c>
       <c r="B58">
-        <v>1.373448064608722E-2</v>
+        <v>0.01373448064608722</v>
       </c>
       <c r="C58">
-        <v>1.264275945277245E-3</v>
+        <v>0.001264275945277245</v>
       </c>
       <c r="D58">
-        <v>3.9333708464405724E-3</v>
+        <v>0.003933370846440572</v>
       </c>
       <c r="E58">
-        <v>0.39257985317688421</v>
+        <v>0.3925798531768842</v>
       </c>
       <c r="F58">
-        <v>0.40075245277459309</v>
+        <v>0.4007524527745931</v>
       </c>
       <c r="G58">
-        <v>9.2873434090823461E-3</v>
+        <v>0.009287343409082346</v>
       </c>
       <c r="H58">
         <v>21</v>
@@ -3152,45 +3131,45 @@
         <v>12</v>
       </c>
       <c r="J58">
-        <v>7.2263439682269572</v>
+        <v>7.226343968226957</v>
       </c>
       <c r="K58">
-        <v>0.34083626765051689</v>
+        <v>0.3408362676505169</v>
       </c>
       <c r="L58">
-        <v>1.9101405049998459</v>
+        <v>1.910140504999846</v>
       </c>
       <c r="M58">
-        <v>6.3359830042053283E-2</v>
+        <v>0.06335983004205328</v>
       </c>
       <c r="N58">
         <v>0.4222201631023329</v>
       </c>
       <c r="O58">
-        <v>0.27995273704547657</v>
-      </c>
-    </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.2799527370454766</v>
+      </c>
+    </row>
+    <row r="59" spans="1:15">
       <c r="A59" s="2">
         <v>45569</v>
       </c>
       <c r="B59">
-        <v>8.6616702605087238E-3</v>
+        <v>0.008661670260508724</v>
       </c>
       <c r="C59">
-        <v>-1.769720507879598E-3</v>
+        <v>-0.001769720507879598</v>
       </c>
       <c r="D59">
-        <v>1.6363363679525701E-3</v>
+        <v>0.00163633636795257</v>
       </c>
       <c r="E59">
-        <v>0.34031801177312232</v>
+        <v>0.3403180117731223</v>
       </c>
       <c r="F59">
-        <v>-0.64684893497077012</v>
+        <v>-0.6468489349707701</v>
       </c>
       <c r="G59">
-        <v>6.2506100504224364E-3</v>
+        <v>0.006250610050422436</v>
       </c>
       <c r="H59">
         <v>10</v>
@@ -3199,45 +3178,45 @@
         <v>4</v>
       </c>
       <c r="J59">
-        <v>3.5939646731105559</v>
+        <v>3.593964673110556</v>
       </c>
       <c r="K59">
         <v>0</v>
       </c>
       <c r="L59">
-        <v>1.8949467468918251</v>
+        <v>1.894946746891825</v>
       </c>
       <c r="M59">
-        <v>6.4006522267039387E-2</v>
+        <v>0.06400652226703939</v>
       </c>
       <c r="N59">
-        <v>0.21688813561432291</v>
+        <v>0.2168881356143229</v>
       </c>
       <c r="O59">
-        <v>0.24559763205557261</v>
-      </c>
-    </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.2455976320555726</v>
+      </c>
+    </row>
+    <row r="60" spans="1:15">
       <c r="A60" s="2">
         <v>45597</v>
       </c>
       <c r="B60">
-        <v>1.4858324353333389E-2</v>
+        <v>0.01485832435333339</v>
       </c>
       <c r="C60">
-        <v>-1.4908367055045809E-3</v>
+        <v>-0.001490836705504581</v>
       </c>
       <c r="D60">
-        <v>4.0783234986294927E-3</v>
+        <v>0.004078323498629493</v>
       </c>
       <c r="E60">
-        <v>-9.1215633758161052E-2</v>
+        <v>-0.09121563375816105</v>
       </c>
       <c r="F60">
-        <v>0.47906936391656041</v>
+        <v>0.4790693639165604</v>
       </c>
       <c r="G60">
-        <v>1.0527635717434151E-2</v>
+        <v>0.01052763571743415</v>
       </c>
       <c r="H60">
         <v>23</v>
@@ -3246,45 +3225,45 @@
         <v>15</v>
       </c>
       <c r="J60">
-        <v>8.1889734942418748</v>
+        <v>8.188973494241875</v>
       </c>
       <c r="K60">
         <v>0.4406364311206537</v>
       </c>
       <c r="L60">
-        <v>1.6635629738730751</v>
+        <v>1.663562973873075</v>
       </c>
       <c r="M60">
-        <v>6.929682093568329E-2</v>
+        <v>0.06929682093568329</v>
       </c>
       <c r="N60">
         <v>0.2344167395234216</v>
       </c>
       <c r="O60">
-        <v>0.24802057374031411</v>
-      </c>
-    </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.2480205737403141</v>
+      </c>
+    </row>
+    <row r="61" spans="1:15">
       <c r="A61" s="2">
         <v>45632</v>
       </c>
       <c r="B61">
-        <v>1.151767949383576E-2</v>
+        <v>0.01151767949383576</v>
       </c>
       <c r="C61">
-        <v>2.0044825005475892E-3</v>
+        <v>0.002004482500547589</v>
       </c>
       <c r="D61">
-        <v>3.3846878387486482E-3</v>
+        <v>0.003384687838748648</v>
       </c>
       <c r="E61">
-        <v>-0.34059016697155181</v>
+        <v>-0.3405901669715518</v>
       </c>
       <c r="F61">
         <v>-0.1018102446209054</v>
       </c>
       <c r="G61">
-        <v>8.7293774970506506E-3</v>
+        <v>0.008729377497050651</v>
       </c>
       <c r="H61">
         <v>18</v>
@@ -3296,42 +3275,42 @@
         <v>5.564262701001855</v>
       </c>
       <c r="K61">
-        <v>0.18894089762385519</v>
+        <v>0.1889408976238552</v>
       </c>
       <c r="L61">
-        <v>1.6455868606584401</v>
+        <v>1.64558686065844</v>
       </c>
       <c r="M61">
-        <v>6.7681522920317136E-2</v>
+        <v>0.06768152292031714</v>
       </c>
       <c r="N61">
-        <v>0.32817607401741861</v>
+        <v>0.3281760740174186</v>
       </c>
       <c r="O61">
-        <v>0.29145727698606172</v>
-      </c>
-    </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.2914572769860617</v>
+      </c>
+    </row>
+    <row r="62" spans="1:15">
       <c r="A62" s="2">
         <v>45660</v>
       </c>
       <c r="B62">
-        <v>1.0492207030389439E-2</v>
+        <v>0.01049220703038944</v>
       </c>
       <c r="C62">
-        <v>1.2688129698580049E-3</v>
+        <v>0.001268812969858005</v>
       </c>
       <c r="D62">
-        <v>2.384452634056798E-3</v>
+        <v>0.002384452634056798</v>
       </c>
       <c r="E62">
-        <v>0.34697280799074781</v>
+        <v>0.3469728079907478</v>
       </c>
       <c r="F62">
-        <v>0.72938885116681429</v>
+        <v>0.7293888511668143</v>
       </c>
       <c r="G62">
-        <v>7.2192231823095887E-3</v>
+        <v>0.007219223182309589</v>
       </c>
       <c r="H62">
         <v>15</v>
@@ -3340,36 +3319,36 @@
         <v>6</v>
       </c>
       <c r="J62">
-        <v>4.5507814488506408</v>
+        <v>4.550781448850641</v>
       </c>
       <c r="K62">
-        <v>9.1753540789651686E-2</v>
+        <v>0.09175354078965169</v>
       </c>
       <c r="L62">
-        <v>2.0328009849840778</v>
+        <v>2.032800984984078</v>
       </c>
       <c r="M62">
-        <v>5.3725621843131968E-2</v>
+        <v>0.05372562184313197</v>
       </c>
       <c r="N62">
         <v>0.1143706664047769</v>
       </c>
       <c r="O62">
-        <v>0.20670186331225751</v>
-      </c>
-    </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.2067018633122575</v>
+      </c>
+    </row>
+    <row r="63" spans="1:15">
       <c r="A63" s="2">
         <v>45689</v>
       </c>
       <c r="B63">
-        <v>1.6306104741740782E-2</v>
+        <v>0.01630610474174078</v>
       </c>
       <c r="C63">
-        <v>-2.230524630146434E-3</v>
+        <v>-0.002230524630146434</v>
       </c>
       <c r="D63">
-        <v>6.1775030476248667E-3</v>
+        <v>0.006177503047624867</v>
       </c>
       <c r="E63">
         <v>0.1633944368966285</v>
@@ -3378,7 +3357,7 @@
         <v>-0.1837761795827843</v>
       </c>
       <c r="G63">
-        <v>7.1433314456045751E-3</v>
+        <v>0.007143331445604575</v>
       </c>
       <c r="H63">
         <v>25</v>
@@ -3387,45 +3366,45 @@
         <v>6</v>
       </c>
       <c r="J63">
-        <v>7.5485911964734056</v>
+        <v>7.548591196473406</v>
       </c>
       <c r="K63">
-        <v>0.37922724101336058</v>
+        <v>0.3792272410133606</v>
       </c>
       <c r="L63">
         <v>2.224990143501095</v>
       </c>
       <c r="M63">
-        <v>4.8864338545392391E-2</v>
+        <v>0.04886433854539239</v>
       </c>
       <c r="N63">
         <v>0.1665395339046952</v>
       </c>
       <c r="O63">
-        <v>0.19689032402207521</v>
-      </c>
-    </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.1968903240220752</v>
+      </c>
+    </row>
+    <row r="64" spans="1:15">
       <c r="A64" s="2">
         <v>45723</v>
       </c>
       <c r="B64">
-        <v>8.6616702605087238E-3</v>
+        <v>0.008661670260508724</v>
       </c>
       <c r="C64">
-        <v>5.9273850604240447E-4</v>
+        <v>0.0005927385060424045</v>
       </c>
       <c r="D64">
-        <v>1.6363363679525701E-3</v>
+        <v>0.00163633636795257</v>
       </c>
       <c r="E64">
-        <v>6.1765221276997517E-2</v>
+        <v>0.06176522127699752</v>
       </c>
       <c r="F64">
-        <v>8.1169295258283994E-2</v>
+        <v>0.08116929525828399</v>
       </c>
       <c r="G64">
-        <v>1.1572808838609051E-2</v>
+        <v>0.01157280883860905</v>
       </c>
       <c r="H64">
         <v>10</v>
@@ -3443,36 +3422,36 @@
         <v>2.071183125017892</v>
       </c>
       <c r="M64">
-        <v>5.0802313100858962E-2</v>
+        <v>0.05080231310085896</v>
       </c>
       <c r="N64">
-        <v>0.17781361768167539</v>
+        <v>0.1778136176816754</v>
       </c>
       <c r="O64">
-        <v>0.19077917012121259</v>
-      </c>
-    </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.1907791701212126</v>
+      </c>
+    </row>
+    <row r="65" spans="1:15">
       <c r="A65" s="2">
         <v>45751</v>
       </c>
       <c r="B65">
-        <v>1.586543592776116E-2</v>
+        <v>0.01586543592776116</v>
       </c>
       <c r="C65">
-        <v>-4.3397589413729688E-4</v>
+        <v>-0.0004339758941372969</v>
       </c>
       <c r="D65">
-        <v>6.6225341766122311E-3</v>
+        <v>0.006622534176612231</v>
       </c>
       <c r="E65">
-        <v>-0.68643587479847068</v>
+        <v>-0.6864358747984707</v>
       </c>
       <c r="F65">
-        <v>0.95903704459251138</v>
+        <v>0.9590370445925114</v>
       </c>
       <c r="G65">
-        <v>9.6783363996669688E-3</v>
+        <v>0.009678336399666969</v>
       </c>
       <c r="H65">
         <v>24</v>
@@ -3481,16 +3460,16 @@
         <v>13</v>
       </c>
       <c r="J65">
-        <v>6.9785397280277719</v>
+        <v>6.978539728027772</v>
       </c>
       <c r="K65">
-        <v>0.33424430602966398</v>
+        <v>0.334244306029664</v>
       </c>
       <c r="L65">
-        <v>2.2795714813342611</v>
+        <v>2.279571481334261</v>
       </c>
       <c r="M65">
-        <v>4.6618842014556947E-2</v>
+        <v>0.04661884201455695</v>
       </c>
       <c r="N65">
         <v>0.2447654705520679</v>
@@ -3499,27 +3478,27 @@
         <v>0.2184948640366601</v>
       </c>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:15">
       <c r="A66" s="2">
         <v>45779</v>
       </c>
       <c r="B66">
-        <v>9.818066175472347E-3</v>
+        <v>0.009818066175472347</v>
       </c>
       <c r="C66">
-        <v>1.06876388039743E-3</v>
+        <v>0.00106876388039743</v>
       </c>
       <c r="D66">
-        <v>2.1409898008459328E-3</v>
+        <v>0.002140989800845933</v>
       </c>
       <c r="E66">
-        <v>-0.20619481683849189</v>
+        <v>-0.2061948168384919</v>
       </c>
       <c r="F66">
-        <v>0.32664383770935018</v>
+        <v>0.3266438377093502</v>
       </c>
       <c r="G66">
-        <v>1.149749764181043E-2</v>
+        <v>0.01149749764181043</v>
       </c>
       <c r="H66">
         <v>14</v>
@@ -3528,16 +3507,16 @@
         <v>18</v>
       </c>
       <c r="J66">
-        <v>4.3994754991814249</v>
+        <v>4.399475499181425</v>
       </c>
       <c r="K66">
-        <v>9.0471159305983262E-2</v>
+        <v>0.09047115930598326</v>
       </c>
       <c r="L66">
         <v>2.38496757041804</v>
       </c>
       <c r="M66">
-        <v>4.3735700153457853E-2</v>
+        <v>0.04373570015345785</v>
       </c>
       <c r="N66">
         <v>0.1031353453530021</v>
@@ -3546,27 +3525,27 @@
         <v>0.1672988402042267</v>
       </c>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:15">
       <c r="A67" s="2">
         <v>45814</v>
       </c>
       <c r="B67">
-        <v>1.0160170570047139E-2</v>
+        <v>0.01016017057004714</v>
       </c>
       <c r="C67">
-        <v>9.8971469274579458E-4</v>
+        <v>0.0009897146927457946</v>
       </c>
       <c r="D67">
-        <v>2.0194674305135212E-3</v>
+        <v>0.002019467430513521</v>
       </c>
       <c r="E67">
-        <v>-0.29824518092638702</v>
+        <v>-0.298245180926387</v>
       </c>
       <c r="F67">
-        <v>9.2848426609035417E-3</v>
+        <v>0.009284842660903542</v>
       </c>
       <c r="G67">
-        <v>6.2871264652626614E-3</v>
+        <v>0.006287126465262661</v>
       </c>
       <c r="H67">
         <v>15</v>
@@ -3575,45 +3554,45 @@
         <v>4</v>
       </c>
       <c r="J67">
-        <v>4.7372398901567241</v>
+        <v>4.737239890156724</v>
       </c>
       <c r="K67">
-        <v>0.13109649732295969</v>
+        <v>0.1310964973229597</v>
       </c>
       <c r="L67">
-        <v>2.8838636405106861</v>
+        <v>2.883863640510686</v>
       </c>
       <c r="M67">
-        <v>3.3088248501350191E-2</v>
+        <v>0.03308824850135019</v>
       </c>
       <c r="N67">
         <v>0.1303567606353446</v>
       </c>
       <c r="O67">
-        <v>0.14698407622958651</v>
-      </c>
-    </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.1469840762295865</v>
+      </c>
+    </row>
+    <row r="68" spans="1:15">
       <c r="A68" s="2">
         <v>45842</v>
       </c>
       <c r="B68">
-        <v>1.038127079803871E-2</v>
+        <v>0.01038127079803871</v>
       </c>
       <c r="C68">
-        <v>6.3524724714465568E-4</v>
+        <v>0.0006352472471446557</v>
       </c>
       <c r="D68">
-        <v>2.3693535760444329E-3</v>
+        <v>0.002369353576044433</v>
       </c>
       <c r="E68">
-        <v>-0.10564278697989769</v>
+        <v>-0.1056427869798977</v>
       </c>
       <c r="F68">
-        <v>-3.7927014293490269E-2</v>
+        <v>-0.03792701429349027</v>
       </c>
       <c r="G68">
-        <v>5.1844394441163894E-3</v>
+        <v>0.005184439444116389</v>
       </c>
       <c r="H68">
         <v>15</v>
@@ -3622,45 +3601,45 @@
         <v>2</v>
       </c>
       <c r="J68">
-        <v>4.3311443947290096</v>
+        <v>4.33114439472901</v>
       </c>
       <c r="K68">
-        <v>9.5018416764556912E-2</v>
+        <v>0.09501841676455691</v>
       </c>
       <c r="L68">
         <v>1.784295230373802</v>
       </c>
       <c r="M68">
-        <v>5.9120552876371829E-2</v>
+        <v>0.05912055287637183</v>
       </c>
       <c r="N68">
-        <v>9.3750533808613923E-2</v>
+        <v>0.09375053380861392</v>
       </c>
       <c r="O68">
         <v>0.1209112938116014</v>
       </c>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:15">
       <c r="A69" s="2">
         <v>45870</v>
       </c>
       <c r="B69">
-        <v>1.3045572481326749E-2</v>
+        <v>0.01304557248132675</v>
       </c>
       <c r="C69">
-        <v>1.0996660193533651E-3</v>
+        <v>0.001099666019353365</v>
       </c>
       <c r="D69">
-        <v>5.1880835930378398E-3</v>
+        <v>0.00518808359303784</v>
       </c>
       <c r="E69">
-        <v>0.55688025101336325</v>
+        <v>0.5568802510133632</v>
       </c>
       <c r="F69">
-        <v>0.49787240121745252</v>
+        <v>0.4978724012174525</v>
       </c>
       <c r="G69">
-        <v>6.4303926875014161E-3</v>
+        <v>0.006430392687501416</v>
       </c>
       <c r="H69">
         <v>20</v>
@@ -3669,45 +3648,45 @@
         <v>4</v>
       </c>
       <c r="J69">
-        <v>5.7324569257349891</v>
+        <v>5.732456925734989</v>
       </c>
       <c r="K69">
-        <v>0.25098635036537398</v>
+        <v>0.250986350365374</v>
       </c>
       <c r="L69">
-        <v>1.7265962872784359</v>
+        <v>1.726596287278436</v>
       </c>
       <c r="M69">
-        <v>5.9999610758361431E-2</v>
+        <v>0.05999961075836143</v>
       </c>
       <c r="N69">
-        <v>0.33280474318333347</v>
+        <v>0.3328047431833335</v>
       </c>
       <c r="O69">
-        <v>0.22071612476556329</v>
-      </c>
-    </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.2207161247655633</v>
+      </c>
+    </row>
+    <row r="70" spans="1:15">
       <c r="A70" s="2">
         <v>45905</v>
       </c>
       <c r="B70">
-        <v>1.8138146681774981E-2</v>
+        <v>0.01813814668177498</v>
       </c>
       <c r="C70">
-        <v>-2.142981920085768E-3</v>
+        <v>-0.002142981920085768</v>
       </c>
       <c r="D70">
-        <v>8.6360517471025938E-3</v>
+        <v>0.008636051747102594</v>
       </c>
       <c r="E70">
         <v>0.2338228514854733</v>
       </c>
       <c r="F70">
-        <v>-5.8229639785509241E-2</v>
+        <v>-0.05822963978550924</v>
       </c>
       <c r="G70">
-        <v>4.0961505817649546E-3</v>
+        <v>0.004096150581764955</v>
       </c>
       <c r="H70">
         <v>26</v>
@@ -3716,26 +3695,25 @@
         <v>1</v>
       </c>
       <c r="J70">
-        <v>8.0702927237776692</v>
+        <v>8.070292723777669</v>
       </c>
       <c r="K70">
         <v>0.5071992593039466</v>
       </c>
       <c r="L70">
-        <v>1.5273848523209741</v>
+        <v>1.527384852320974</v>
       </c>
       <c r="M70">
-        <v>6.4024335714634617E-2</v>
+        <v>0.06402433571463462</v>
       </c>
       <c r="N70">
-        <v>0.25825190339164611</v>
+        <v>0.2582519033916461</v>
       </c>
       <c r="O70">
-        <v>0.25288617326959162</v>
+        <v>0.2528861732695916</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>